<commit_message>
Add read_workbook_cells and update_workbook tools to agent
Allows the agent to read and write any cell in any sheet of the
workbook via chat. Enables persistent changes to assignments, dates,
priorities, hours, and any other field without manual Excel editing.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ETE PMO Resource Planner.xlsx
+++ b/ETE PMO Resource Planner.xlsx
@@ -8876,12 +8876,12 @@
       </c>
       <c r="H26" s="282" t="inlineStr">
         <is>
-          <t>2025-11-17</t>
+          <t>11/17/2025</t>
         </is>
       </c>
       <c r="I26" s="282" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>04/24/2026</t>
         </is>
       </c>
     </row>
@@ -8915,12 +8915,12 @@
       </c>
       <c r="H27" s="282" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>02/23/2026</t>
         </is>
       </c>
       <c r="I27" s="282" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>04/17/2026</t>
         </is>
       </c>
     </row>
@@ -8954,12 +8954,12 @@
       </c>
       <c r="H28" s="282" t="inlineStr">
         <is>
-          <t>2025-10-14</t>
+          <t>10/14/2025</t>
         </is>
       </c>
       <c r="I28" s="282" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>06/01/2026</t>
         </is>
       </c>
     </row>
@@ -8993,12 +8993,12 @@
       </c>
       <c r="H29" s="282" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>02/15/2026</t>
         </is>
       </c>
       <c r="I29" s="282" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>06/30/2026</t>
         </is>
       </c>
     </row>
@@ -11206,7 +11206,11 @@
           <t>Systems Applications</t>
         </is>
       </c>
-      <c r="M4" s="93" t="n"/>
+      <c r="M4" s="93" t="inlineStr">
+        <is>
+          <t>Emily Fridley</t>
+        </is>
+      </c>
       <c r="N4" s="93" t="inlineStr">
         <is>
           <t>Jim Young</t>
@@ -19000,7 +19004,7 @@
     <row r="2">
       <c r="A2" s="271" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-31  |  Color = priority</t>
+          <t>Generated: 03/31/2026  |  Color = priority</t>
         </is>
       </c>
     </row>
@@ -19403,12 +19407,12 @@
       </c>
       <c r="E9" s="275" t="inlineStr">
         <is>
-          <t>2025-11-17</t>
+          <t>11/17/2025</t>
         </is>
       </c>
       <c r="F9" s="275" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>04/24/2026</t>
         </is>
       </c>
       <c r="G9" s="275" t="inlineStr">
@@ -19461,12 +19465,12 @@
       </c>
       <c r="E10" s="275" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>02/23/2026</t>
         </is>
       </c>
       <c r="F10" s="275" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>04/17/2026</t>
         </is>
       </c>
       <c r="G10" s="275" t="inlineStr">
@@ -19504,12 +19508,12 @@
       </c>
       <c r="E11" s="275" t="inlineStr">
         <is>
-          <t>2025-10-14</t>
+          <t>10/14/2025</t>
         </is>
       </c>
       <c r="F11" s="275" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>06/01/2026</t>
         </is>
       </c>
       <c r="G11" s="275" t="inlineStr">
@@ -19573,12 +19577,12 @@
       </c>
       <c r="E12" s="275" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>03/03/2026</t>
         </is>
       </c>
       <c r="F12" s="275" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>03/13/2026</t>
         </is>
       </c>
       <c r="G12" s="275" t="inlineStr">
@@ -19610,12 +19614,12 @@
       </c>
       <c r="E13" s="275" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>02/15/2026</t>
         </is>
       </c>
       <c r="F13" s="275" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>06/30/2026</t>
         </is>
       </c>
       <c r="G13" s="275" t="inlineStr">

</xml_diff>

<commit_message>
Add Developer person assignment column (Q) to Portfolio
Insert column Q between Technical (P) and T-Shirt Size (now R).
Update all column indices in excel_connector.py (17+ shifted by 1).
Add Developer to _ASSIGNMENT_COLUMNS for read_assignments().
Assign Emily Fridley (PM), Audrey Debaere (BA), Alex Young (Developer)
to all 15 active projects for heatmap testing.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ETE PMO Resource Planner.xlsx
+++ b/ETE PMO Resource Planner.xlsx
@@ -8751,7 +8751,9 @@
       <c r="E23" s="304" t="n">
         <v>220</v>
       </c>
-      <c r="F23" s="282" t="n"/>
+      <c r="F23" s="282" t="n">
+        <v/>
+      </c>
       <c r="G23" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -8790,7 +8792,9 @@
       <c r="E24" s="282" t="n">
         <v>40</v>
       </c>
-      <c r="F24" s="282" t="n"/>
+      <c r="F24" s="282" t="n">
+        <v/>
+      </c>
       <c r="G24" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -8829,7 +8833,9 @@
       <c r="E25" s="304" t="n">
         <v>170</v>
       </c>
-      <c r="F25" s="282" t="n"/>
+      <c r="F25" s="282" t="n">
+        <v/>
+      </c>
       <c r="G25" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -8868,7 +8874,9 @@
       <c r="E26" s="304" t="n">
         <v>544</v>
       </c>
-      <c r="F26" s="282" t="n"/>
+      <c r="F26" s="282" t="n">
+        <v/>
+      </c>
       <c r="G26" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -8907,7 +8915,9 @@
       <c r="E27" s="282" t="n">
         <v>120</v>
       </c>
-      <c r="F27" s="282" t="n"/>
+      <c r="F27" s="282" t="n">
+        <v/>
+      </c>
       <c r="G27" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -8946,7 +8956,9 @@
       <c r="E28" s="304" t="n">
         <v>148</v>
       </c>
-      <c r="F28" s="282" t="n"/>
+      <c r="F28" s="282" t="n">
+        <v/>
+      </c>
       <c r="G28" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -8985,7 +8997,9 @@
       <c r="E29" s="304" t="n">
         <v>84</v>
       </c>
-      <c r="F29" s="282" t="n"/>
+      <c r="F29" s="282" t="n">
+        <v/>
+      </c>
       <c r="G29" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -9024,7 +9038,9 @@
       <c r="E30" s="304" t="n">
         <v>170</v>
       </c>
-      <c r="F30" s="282" t="n"/>
+      <c r="F30" s="282" t="n">
+        <v/>
+      </c>
       <c r="G30" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -9063,7 +9079,9 @@
       <c r="E31" s="304" t="n">
         <v>204</v>
       </c>
-      <c r="F31" s="282" t="n"/>
+      <c r="F31" s="282" t="n">
+        <v/>
+      </c>
       <c r="G31" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -9102,7 +9120,9 @@
       <c r="E32" s="282" t="n">
         <v>640</v>
       </c>
-      <c r="F32" s="282" t="n"/>
+      <c r="F32" s="282" t="n">
+        <v/>
+      </c>
       <c r="G32" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -9141,7 +9161,9 @@
       <c r="E33" s="282" t="n">
         <v>120</v>
       </c>
-      <c r="F33" s="282" t="n"/>
+      <c r="F33" s="282" t="n">
+        <v/>
+      </c>
       <c r="G33" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -9180,7 +9202,9 @@
       <c r="E34" s="304" t="n">
         <v>34</v>
       </c>
-      <c r="F34" s="282" t="n"/>
+      <c r="F34" s="282" t="n">
+        <v/>
+      </c>
       <c r="G34" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -9993,15 +10017,33 @@
       <c r="C22" s="282" t="n">
         <v>200</v>
       </c>
-      <c r="D22" s="282" t="n"/>
-      <c r="E22" s="290" t="n"/>
-      <c r="F22" s="290" t="n"/>
-      <c r="G22" s="290" t="n"/>
-      <c r="H22" s="290" t="n"/>
-      <c r="I22" s="290" t="n"/>
-      <c r="J22" s="290" t="n"/>
-      <c r="K22" s="290" t="n"/>
-      <c r="L22" s="290" t="n"/>
+      <c r="D22" s="282" t="n">
+        <v/>
+      </c>
+      <c r="E22" s="290" t="n">
+        <v/>
+      </c>
+      <c r="F22" s="290" t="n">
+        <v/>
+      </c>
+      <c r="G22" s="290" t="n">
+        <v/>
+      </c>
+      <c r="H22" s="290" t="n">
+        <v/>
+      </c>
+      <c r="I22" s="290" t="n">
+        <v/>
+      </c>
+      <c r="J22" s="290" t="n">
+        <v/>
+      </c>
+      <c r="K22" s="290" t="n">
+        <v/>
+      </c>
+      <c r="L22" s="290" t="n">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="287" t="inlineStr">
@@ -10017,15 +10059,33 @@
       <c r="C23" s="282" t="n">
         <v>40</v>
       </c>
-      <c r="D23" s="282" t="n"/>
-      <c r="E23" s="290" t="n"/>
-      <c r="F23" s="290" t="n"/>
-      <c r="G23" s="290" t="n"/>
-      <c r="H23" s="290" t="n"/>
-      <c r="I23" s="290" t="n"/>
-      <c r="J23" s="290" t="n"/>
-      <c r="K23" s="290" t="n"/>
-      <c r="L23" s="290" t="n"/>
+      <c r="D23" s="282" t="n">
+        <v/>
+      </c>
+      <c r="E23" s="290" t="n">
+        <v/>
+      </c>
+      <c r="F23" s="290" t="n">
+        <v/>
+      </c>
+      <c r="G23" s="290" t="n">
+        <v/>
+      </c>
+      <c r="H23" s="290" t="n">
+        <v/>
+      </c>
+      <c r="I23" s="290" t="n">
+        <v/>
+      </c>
+      <c r="J23" s="290" t="n">
+        <v/>
+      </c>
+      <c r="K23" s="290" t="n">
+        <v/>
+      </c>
+      <c r="L23" s="290" t="n">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="287" t="inlineStr">
@@ -10041,15 +10101,33 @@
       <c r="C24" s="282" t="n">
         <v>200</v>
       </c>
-      <c r="D24" s="282" t="n"/>
-      <c r="E24" s="290" t="n"/>
-      <c r="F24" s="290" t="n"/>
-      <c r="G24" s="290" t="n"/>
-      <c r="H24" s="290" t="n"/>
-      <c r="I24" s="290" t="n"/>
-      <c r="J24" s="290" t="n"/>
-      <c r="K24" s="290" t="n"/>
-      <c r="L24" s="290" t="n"/>
+      <c r="D24" s="282" t="n">
+        <v/>
+      </c>
+      <c r="E24" s="290" t="n">
+        <v/>
+      </c>
+      <c r="F24" s="290" t="n">
+        <v/>
+      </c>
+      <c r="G24" s="290" t="n">
+        <v/>
+      </c>
+      <c r="H24" s="290" t="n">
+        <v/>
+      </c>
+      <c r="I24" s="290" t="n">
+        <v/>
+      </c>
+      <c r="J24" s="290" t="n">
+        <v/>
+      </c>
+      <c r="K24" s="290" t="n">
+        <v/>
+      </c>
+      <c r="L24" s="290" t="n">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="287" t="inlineStr">
@@ -10065,15 +10143,33 @@
       <c r="C25" s="282" t="n">
         <v>640</v>
       </c>
-      <c r="D25" s="282" t="n"/>
-      <c r="E25" s="290" t="n"/>
-      <c r="F25" s="290" t="n"/>
-      <c r="G25" s="290" t="n"/>
-      <c r="H25" s="290" t="n"/>
-      <c r="I25" s="290" t="n"/>
-      <c r="J25" s="290" t="n"/>
-      <c r="K25" s="290" t="n"/>
-      <c r="L25" s="290" t="n"/>
+      <c r="D25" s="282" t="n">
+        <v/>
+      </c>
+      <c r="E25" s="290" t="n">
+        <v/>
+      </c>
+      <c r="F25" s="290" t="n">
+        <v/>
+      </c>
+      <c r="G25" s="290" t="n">
+        <v/>
+      </c>
+      <c r="H25" s="290" t="n">
+        <v/>
+      </c>
+      <c r="I25" s="290" t="n">
+        <v/>
+      </c>
+      <c r="J25" s="290" t="n">
+        <v/>
+      </c>
+      <c r="K25" s="290" t="n">
+        <v/>
+      </c>
+      <c r="L25" s="290" t="n">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="287" t="inlineStr">
@@ -10089,15 +10185,33 @@
       <c r="C26" s="282" t="n">
         <v>120</v>
       </c>
-      <c r="D26" s="282" t="n"/>
-      <c r="E26" s="290" t="n"/>
-      <c r="F26" s="290" t="n"/>
-      <c r="G26" s="290" t="n"/>
-      <c r="H26" s="290" t="n"/>
-      <c r="I26" s="290" t="n"/>
-      <c r="J26" s="290" t="n"/>
-      <c r="K26" s="290" t="n"/>
-      <c r="L26" s="290" t="n"/>
+      <c r="D26" s="282" t="n">
+        <v/>
+      </c>
+      <c r="E26" s="290" t="n">
+        <v/>
+      </c>
+      <c r="F26" s="290" t="n">
+        <v/>
+      </c>
+      <c r="G26" s="290" t="n">
+        <v/>
+      </c>
+      <c r="H26" s="290" t="n">
+        <v/>
+      </c>
+      <c r="I26" s="290" t="n">
+        <v/>
+      </c>
+      <c r="J26" s="290" t="n">
+        <v/>
+      </c>
+      <c r="K26" s="290" t="n">
+        <v/>
+      </c>
+      <c r="L26" s="290" t="n">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="287" t="inlineStr">
@@ -10113,15 +10227,33 @@
       <c r="C27" s="282" t="n">
         <v>1480</v>
       </c>
-      <c r="D27" s="282" t="n"/>
-      <c r="E27" s="290" t="n"/>
-      <c r="F27" s="290" t="n"/>
-      <c r="G27" s="290" t="n"/>
-      <c r="H27" s="290" t="n"/>
-      <c r="I27" s="290" t="n"/>
-      <c r="J27" s="290" t="n"/>
-      <c r="K27" s="290" t="n"/>
-      <c r="L27" s="290" t="n"/>
+      <c r="D27" s="282" t="n">
+        <v/>
+      </c>
+      <c r="E27" s="290" t="n">
+        <v/>
+      </c>
+      <c r="F27" s="290" t="n">
+        <v/>
+      </c>
+      <c r="G27" s="290" t="n">
+        <v/>
+      </c>
+      <c r="H27" s="290" t="n">
+        <v/>
+      </c>
+      <c r="I27" s="290" t="n">
+        <v/>
+      </c>
+      <c r="J27" s="290" t="n">
+        <v/>
+      </c>
+      <c r="K27" s="290" t="n">
+        <v/>
+      </c>
+      <c r="L27" s="290" t="n">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="287" t="inlineStr">
@@ -10137,15 +10269,33 @@
       <c r="C28" s="282" t="n">
         <v>240</v>
       </c>
-      <c r="D28" s="282" t="n"/>
-      <c r="E28" s="290" t="n"/>
-      <c r="F28" s="290" t="n"/>
-      <c r="G28" s="290" t="n"/>
-      <c r="H28" s="290" t="n"/>
-      <c r="I28" s="290" t="n"/>
-      <c r="J28" s="290" t="n"/>
-      <c r="K28" s="290" t="n"/>
-      <c r="L28" s="290" t="n"/>
+      <c r="D28" s="282" t="n">
+        <v/>
+      </c>
+      <c r="E28" s="290" t="n">
+        <v/>
+      </c>
+      <c r="F28" s="290" t="n">
+        <v/>
+      </c>
+      <c r="G28" s="290" t="n">
+        <v/>
+      </c>
+      <c r="H28" s="290" t="n">
+        <v/>
+      </c>
+      <c r="I28" s="290" t="n">
+        <v/>
+      </c>
+      <c r="J28" s="290" t="n">
+        <v/>
+      </c>
+      <c r="K28" s="290" t="n">
+        <v/>
+      </c>
+      <c r="L28" s="290" t="n">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="287" t="inlineStr">
@@ -10161,15 +10311,33 @@
       <c r="C29" s="282" t="n">
         <v>200</v>
       </c>
-      <c r="D29" s="282" t="n"/>
-      <c r="E29" s="290" t="n"/>
-      <c r="F29" s="290" t="n"/>
-      <c r="G29" s="290" t="n"/>
-      <c r="H29" s="290" t="n"/>
-      <c r="I29" s="290" t="n"/>
-      <c r="J29" s="290" t="n"/>
-      <c r="K29" s="290" t="n"/>
-      <c r="L29" s="290" t="n"/>
+      <c r="D29" s="282" t="n">
+        <v/>
+      </c>
+      <c r="E29" s="290" t="n">
+        <v/>
+      </c>
+      <c r="F29" s="290" t="n">
+        <v/>
+      </c>
+      <c r="G29" s="290" t="n">
+        <v/>
+      </c>
+      <c r="H29" s="290" t="n">
+        <v/>
+      </c>
+      <c r="I29" s="290" t="n">
+        <v/>
+      </c>
+      <c r="J29" s="290" t="n">
+        <v/>
+      </c>
+      <c r="K29" s="290" t="n">
+        <v/>
+      </c>
+      <c r="L29" s="290" t="n">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="287" t="inlineStr">
@@ -10185,15 +10353,33 @@
       <c r="C30" s="282" t="n">
         <v>240</v>
       </c>
-      <c r="D30" s="282" t="n"/>
-      <c r="E30" s="290" t="n"/>
-      <c r="F30" s="290" t="n"/>
-      <c r="G30" s="290" t="n"/>
-      <c r="H30" s="290" t="n"/>
-      <c r="I30" s="290" t="n"/>
-      <c r="J30" s="290" t="n"/>
-      <c r="K30" s="290" t="n"/>
-      <c r="L30" s="290" t="n"/>
+      <c r="D30" s="282" t="n">
+        <v/>
+      </c>
+      <c r="E30" s="290" t="n">
+        <v/>
+      </c>
+      <c r="F30" s="290" t="n">
+        <v/>
+      </c>
+      <c r="G30" s="290" t="n">
+        <v/>
+      </c>
+      <c r="H30" s="290" t="n">
+        <v/>
+      </c>
+      <c r="I30" s="290" t="n">
+        <v/>
+      </c>
+      <c r="J30" s="290" t="n">
+        <v/>
+      </c>
+      <c r="K30" s="290" t="n">
+        <v/>
+      </c>
+      <c r="L30" s="290" t="n">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="287" t="inlineStr">
@@ -10209,15 +10395,33 @@
       <c r="C31" s="282" t="n">
         <v>640</v>
       </c>
-      <c r="D31" s="282" t="n"/>
-      <c r="E31" s="290" t="n"/>
-      <c r="F31" s="290" t="n"/>
-      <c r="G31" s="290" t="n"/>
-      <c r="H31" s="290" t="n"/>
-      <c r="I31" s="290" t="n"/>
-      <c r="J31" s="290" t="n"/>
-      <c r="K31" s="290" t="n"/>
-      <c r="L31" s="290" t="n"/>
+      <c r="D31" s="282" t="n">
+        <v/>
+      </c>
+      <c r="E31" s="290" t="n">
+        <v/>
+      </c>
+      <c r="F31" s="290" t="n">
+        <v/>
+      </c>
+      <c r="G31" s="290" t="n">
+        <v/>
+      </c>
+      <c r="H31" s="290" t="n">
+        <v/>
+      </c>
+      <c r="I31" s="290" t="n">
+        <v/>
+      </c>
+      <c r="J31" s="290" t="n">
+        <v/>
+      </c>
+      <c r="K31" s="290" t="n">
+        <v/>
+      </c>
+      <c r="L31" s="290" t="n">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="287" t="inlineStr">
@@ -10233,15 +10437,33 @@
       <c r="C32" s="282" t="n">
         <v>120</v>
       </c>
-      <c r="D32" s="282" t="n"/>
-      <c r="E32" s="290" t="n"/>
-      <c r="F32" s="290" t="n"/>
-      <c r="G32" s="290" t="n"/>
-      <c r="H32" s="290" t="n"/>
-      <c r="I32" s="290" t="n"/>
-      <c r="J32" s="290" t="n"/>
-      <c r="K32" s="290" t="n"/>
-      <c r="L32" s="290" t="n"/>
+      <c r="D32" s="282" t="n">
+        <v/>
+      </c>
+      <c r="E32" s="290" t="n">
+        <v/>
+      </c>
+      <c r="F32" s="290" t="n">
+        <v/>
+      </c>
+      <c r="G32" s="290" t="n">
+        <v/>
+      </c>
+      <c r="H32" s="290" t="n">
+        <v/>
+      </c>
+      <c r="I32" s="290" t="n">
+        <v/>
+      </c>
+      <c r="J32" s="290" t="n">
+        <v/>
+      </c>
+      <c r="K32" s="290" t="n">
+        <v/>
+      </c>
+      <c r="L32" s="290" t="n">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="287" t="inlineStr">
@@ -10257,15 +10479,33 @@
       <c r="C33" s="282" t="n">
         <v>40</v>
       </c>
-      <c r="D33" s="282" t="n"/>
-      <c r="E33" s="290" t="n"/>
-      <c r="F33" s="290" t="n"/>
-      <c r="G33" s="290" t="n"/>
-      <c r="H33" s="290" t="n"/>
-      <c r="I33" s="290" t="n"/>
-      <c r="J33" s="290" t="n"/>
-      <c r="K33" s="290" t="n"/>
-      <c r="L33" s="290" t="n"/>
+      <c r="D33" s="282" t="n">
+        <v/>
+      </c>
+      <c r="E33" s="290" t="n">
+        <v/>
+      </c>
+      <c r="F33" s="290" t="n">
+        <v/>
+      </c>
+      <c r="G33" s="290" t="n">
+        <v/>
+      </c>
+      <c r="H33" s="290" t="n">
+        <v/>
+      </c>
+      <c r="I33" s="290" t="n">
+        <v/>
+      </c>
+      <c r="J33" s="290" t="n">
+        <v/>
+      </c>
+      <c r="K33" s="290" t="n">
+        <v/>
+      </c>
+      <c r="L33" s="290" t="n">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="273" t="inlineStr">
@@ -10916,7 +11156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC42"/>
+  <dimension ref="A1:AD42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10976,6 +11216,7 @@
       <c r="AA1" s="3" t="n"/>
       <c r="AB1" s="3" t="n"/>
       <c r="AC1" s="3" t="n"/>
+      <c r="AD1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n"/>
@@ -10994,7 +11235,6 @@
       <c r="N2" s="3" t="n"/>
       <c r="O2" s="3" t="n"/>
       <c r="P2" s="3" t="n"/>
-      <c r="Q2" s="3" t="n"/>
       <c r="R2" s="3" t="n"/>
       <c r="S2" s="3" t="n"/>
       <c r="T2" s="3" t="n"/>
@@ -11007,6 +11247,7 @@
       <c r="AA2" s="3" t="n"/>
       <c r="AB2" s="3" t="n"/>
       <c r="AC2" s="3" t="n"/>
+      <c r="AD2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="87" t="inlineStr">
@@ -11089,67 +11330,72 @@
           <t>Technical</t>
         </is>
       </c>
-      <c r="Q3" s="87" t="inlineStr">
+      <c r="Q3" s="88" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="R3" s="87" t="inlineStr">
         <is>
           <t>T-Shirt Size</t>
         </is>
       </c>
-      <c r="R3" s="87" t="inlineStr">
+      <c r="S3" s="87" t="inlineStr">
         <is>
           <t>Est. Hours</t>
         </is>
       </c>
-      <c r="S3" s="88" t="inlineStr">
+      <c r="T3" s="88" t="inlineStr">
         <is>
           <t>Est. Cost Range</t>
         </is>
       </c>
-      <c r="T3" s="88" t="inlineStr">
+      <c r="U3" s="88" t="inlineStr">
         <is>
           <t>BA %</t>
         </is>
       </c>
-      <c r="U3" s="88" t="inlineStr">
+      <c r="V3" s="88" t="inlineStr">
         <is>
           <t>Functional %</t>
         </is>
       </c>
-      <c r="V3" s="88" t="inlineStr">
+      <c r="W3" s="88" t="inlineStr">
         <is>
           <t>Technical %</t>
         </is>
       </c>
-      <c r="W3" s="88" t="inlineStr">
+      <c r="X3" s="88" t="inlineStr">
         <is>
           <t>Developer %</t>
         </is>
       </c>
-      <c r="X3" s="88" t="inlineStr">
+      <c r="Y3" s="88" t="inlineStr">
         <is>
           <t>Infrastructure %</t>
         </is>
       </c>
-      <c r="Y3" s="88" t="inlineStr">
+      <c r="Z3" s="88" t="inlineStr">
         <is>
           <t>DBA %</t>
         </is>
       </c>
-      <c r="Z3" s="88" t="inlineStr">
+      <c r="AA3" s="88" t="inlineStr">
         <is>
           <t>PM %</t>
         </is>
       </c>
-      <c r="AA3" s="88" t="inlineStr">
+      <c r="AB3" s="88" t="inlineStr">
         <is>
           <t>WMS %</t>
         </is>
       </c>
-      <c r="AB3" s="88" t="inlineStr">
+      <c r="AC3" s="88" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="AC3" s="117" t="inlineStr">
+      <c r="AD3" s="117" t="inlineStr">
         <is>
           <t>Sort Order</t>
         </is>
@@ -11213,39 +11459,44 @@
       </c>
       <c r="N4" s="93" t="inlineStr">
         <is>
-          <t>Jim Young</t>
+          <t>Audrey Debaere</t>
         </is>
       </c>
       <c r="O4" s="93" t="n"/>
       <c r="P4" s="93" t="n"/>
-      <c r="Q4" s="89" t="inlineStr">
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Alex Young</t>
+        </is>
+      </c>
+      <c r="R4" s="89" t="inlineStr">
         <is>
           <t>XXL: &gt; 640 Hours</t>
         </is>
       </c>
-      <c r="R4" s="89" t="n">
+      <c r="S4" s="89" t="n">
         <v>1480</v>
       </c>
-      <c r="S4" s="94">
+      <c r="T4" s="94">
         <f>$R4*65</f>
         <v/>
       </c>
-      <c r="T4" s="95" t="n">
+      <c r="U4" s="95" t="n">
         <v>0.1</v>
       </c>
-      <c r="U4" s="95" t="n"/>
       <c r="V4" s="95" t="n"/>
       <c r="W4" s="95" t="n"/>
       <c r="X4" s="95" t="n"/>
       <c r="Y4" s="95" t="n"/>
-      <c r="Z4" s="96" t="n"/>
+      <c r="Z4" s="95" t="n"/>
       <c r="AA4" s="96" t="n"/>
-      <c r="AB4" s="97" t="inlineStr">
+      <c r="AB4" s="96" t="n"/>
+      <c r="AC4" s="97" t="inlineStr">
         <is>
           <t>Completed Q1</t>
         </is>
       </c>
-      <c r="AC4" s="98">
+      <c r="AD4" s="98">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F4)),ISNUMBER(SEARCH("NOT APPROVED",$F4))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F4)),3,1))</f>
         <v/>
       </c>
@@ -11306,35 +11557,44 @@
           <t>Emily Fridley</t>
         </is>
       </c>
-      <c r="N5" s="103" t="n"/>
+      <c r="N5" s="103" t="inlineStr">
+        <is>
+          <t>Audrey Debaere</t>
+        </is>
+      </c>
       <c r="O5" s="103" t="n"/>
       <c r="P5" s="103" t="n"/>
-      <c r="Q5" s="99" t="inlineStr">
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Alex Young</t>
+        </is>
+      </c>
+      <c r="R5" s="99" t="inlineStr">
         <is>
           <t>L: 160-320 Hours</t>
         </is>
       </c>
-      <c r="R5" s="99" t="n">
+      <c r="S5" s="99" t="n">
         <v>240</v>
       </c>
-      <c r="S5" s="104">
+      <c r="T5" s="104">
         <f>$R5*65</f>
         <v/>
       </c>
-      <c r="T5" s="105" t="n">
+      <c r="U5" s="105" t="n">
         <v>0.1</v>
       </c>
-      <c r="U5" s="105" t="n"/>
       <c r="V5" s="105" t="n"/>
       <c r="W5" s="105" t="n"/>
       <c r="X5" s="105" t="n"/>
       <c r="Y5" s="105" t="n"/>
-      <c r="Z5" s="105" t="n">
+      <c r="Z5" s="105" t="n"/>
+      <c r="AA5" s="105" t="n">
         <v>0.25</v>
       </c>
-      <c r="AA5" s="105" t="n"/>
-      <c r="AB5" s="103" t="n"/>
-      <c r="AC5" s="106">
+      <c r="AB5" s="105" t="n"/>
+      <c r="AC5" s="103" t="n"/>
+      <c r="AD5" s="106">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F5)),ISNUMBER(SEARCH("NOT APPROVED",$F5))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F5)),3,1))</f>
         <v/>
       </c>
@@ -11390,10 +11650,14 @@
           <t>Systems Applications</t>
         </is>
       </c>
-      <c r="M6" s="93" t="n"/>
+      <c r="M6" s="93" t="inlineStr">
+        <is>
+          <t>Emily Fridley</t>
+        </is>
+      </c>
       <c r="N6" s="93" t="inlineStr">
         <is>
-          <t>Cristian Varelas</t>
+          <t>Audrey Debaere</t>
         </is>
       </c>
       <c r="O6" s="93" t="n"/>
@@ -11402,32 +11666,37 @@
           <t>Colin Olson</t>
         </is>
       </c>
-      <c r="Q6" s="89" t="inlineStr">
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Alex Young</t>
+        </is>
+      </c>
+      <c r="R6" s="89" t="inlineStr">
         <is>
           <t>XXL: &gt; 640 Hours</t>
         </is>
       </c>
-      <c r="R6" s="89" t="n">
+      <c r="S6" s="89" t="n">
         <v>640</v>
       </c>
-      <c r="S6" s="107">
+      <c r="T6" s="107">
         <f>$R6*65</f>
         <v/>
       </c>
-      <c r="T6" s="96" t="n">
+      <c r="U6" s="96" t="n">
         <v>0.1</v>
       </c>
-      <c r="U6" s="96" t="n"/>
       <c r="V6" s="96" t="n"/>
-      <c r="W6" s="96" t="n">
+      <c r="W6" s="96" t="n"/>
+      <c r="X6" s="96" t="n">
         <v>0.75</v>
       </c>
-      <c r="X6" s="96" t="n"/>
       <c r="Y6" s="96" t="n"/>
       <c r="Z6" s="96" t="n"/>
       <c r="AA6" s="96" t="n"/>
-      <c r="AB6" s="93" t="n"/>
-      <c r="AC6" s="108">
+      <c r="AB6" s="96" t="n"/>
+      <c r="AC6" s="93" t="n"/>
+      <c r="AD6" s="108">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F6)),ISNUMBER(SEARCH("NOT APPROVED",$F6))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F6)),3,1))</f>
         <v/>
       </c>
@@ -11483,30 +11752,43 @@
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="M7" s="93" t="n"/>
-      <c r="N7" s="93" t="n"/>
+      <c r="M7" s="93" t="inlineStr">
+        <is>
+          <t>Emily Fridley</t>
+        </is>
+      </c>
+      <c r="N7" s="93" t="inlineStr">
+        <is>
+          <t>Audrey Debaere</t>
+        </is>
+      </c>
       <c r="O7" s="93" t="n"/>
       <c r="P7" s="93" t="n"/>
-      <c r="Q7" s="89" t="n"/>
-      <c r="R7" s="89" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" s="107">
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Alex Young</t>
+        </is>
+      </c>
+      <c r="R7" s="89" t="n"/>
+      <c r="S7" s="89" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="107">
         <f>$R7*65</f>
         <v/>
       </c>
-      <c r="T7" s="96" t="n">
+      <c r="U7" s="96" t="n">
         <v>0.1</v>
       </c>
-      <c r="U7" s="96" t="n"/>
       <c r="V7" s="96" t="n"/>
       <c r="W7" s="96" t="n"/>
       <c r="X7" s="96" t="n"/>
       <c r="Y7" s="96" t="n"/>
       <c r="Z7" s="96" t="n"/>
       <c r="AA7" s="96" t="n"/>
-      <c r="AB7" s="93" t="n"/>
-      <c r="AC7" s="108">
+      <c r="AB7" s="96" t="n"/>
+      <c r="AC7" s="93" t="n"/>
+      <c r="AD7" s="108">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F7)),ISNUMBER(SEARCH("NOT APPROVED",$F7))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F7)),3,1))</f>
         <v/>
       </c>
@@ -11562,7 +11844,11 @@
           <t>Synnergie</t>
         </is>
       </c>
-      <c r="M8" s="93" t="n"/>
+      <c r="M8" s="93" t="inlineStr">
+        <is>
+          <t>Emily Fridley</t>
+        </is>
+      </c>
       <c r="N8" s="93" t="inlineStr">
         <is>
           <t>Audrey Debaere</t>
@@ -11578,34 +11864,39 @@
           <t>Bhavya Reddy</t>
         </is>
       </c>
-      <c r="Q8" s="89" t="inlineStr">
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Alex Young</t>
+        </is>
+      </c>
+      <c r="R8" s="89" t="inlineStr">
         <is>
           <t>M: 80-160 Hours</t>
         </is>
       </c>
-      <c r="R8" s="89" t="n">
+      <c r="S8" s="89" t="n">
         <v>120</v>
       </c>
-      <c r="S8" s="107">
+      <c r="T8" s="107">
         <f>$R8*65</f>
         <v/>
       </c>
-      <c r="T8" s="96" t="n">
+      <c r="U8" s="96" t="n">
         <v>0.1</v>
       </c>
-      <c r="U8" s="96" t="n">
+      <c r="V8" s="96" t="n">
         <v>0.25</v>
       </c>
-      <c r="V8" s="96" t="n">
+      <c r="W8" s="96" t="n">
         <v>0.65</v>
       </c>
-      <c r="W8" s="96" t="n"/>
       <c r="X8" s="96" t="n"/>
       <c r="Y8" s="96" t="n"/>
       <c r="Z8" s="96" t="n"/>
       <c r="AA8" s="96" t="n"/>
-      <c r="AB8" s="93" t="n"/>
-      <c r="AC8" s="108">
+      <c r="AB8" s="96" t="n"/>
+      <c r="AC8" s="93" t="n"/>
+      <c r="AD8" s="108">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F8)),ISNUMBER(SEARCH("NOT APPROVED",$F8))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F8)),3,1))</f>
         <v/>
       </c>
@@ -11657,41 +11948,47 @@
           <t>Systems Applications</t>
         </is>
       </c>
-      <c r="M9" s="93" t="n"/>
+      <c r="M9" s="93" t="inlineStr">
+        <is>
+          <t>Emily Fridley</t>
+        </is>
+      </c>
       <c r="N9" s="93" t="inlineStr">
         <is>
-          <t>Cristian Varelas</t>
+          <t>Audrey Debaere</t>
         </is>
       </c>
       <c r="O9" s="93" t="n"/>
       <c r="P9" s="93" t="n"/>
-      <c r="Q9" s="89" t="inlineStr">
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Alex Young</t>
+        </is>
+      </c>
+      <c r="R9" s="89" t="inlineStr">
         <is>
           <t>L: 160-320 Hours</t>
         </is>
       </c>
-      <c r="R9" s="89" t="n">
+      <c r="S9" s="89" t="n">
         <v>240</v>
       </c>
-      <c r="S9" s="107">
+      <c r="T9" s="107">
         <f>$R9*65</f>
         <v/>
       </c>
-      <c r="T9" s="109" t="n">
+      <c r="U9" s="109" t="n">
         <v>0.1</v>
       </c>
-      <c r="U9" s="109" t="n">
-        <v>0</v>
-      </c>
       <c r="V9" s="109" t="n">
         <v>0</v>
       </c>
       <c r="W9" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" s="109" t="n">
         <v>0.75</v>
       </c>
-      <c r="X9" s="109" t="n">
-        <v>0</v>
-      </c>
       <c r="Y9" s="109" t="n">
         <v>0</v>
       </c>
@@ -11701,8 +11998,11 @@
       <c r="AA9" s="109" t="n">
         <v>0</v>
       </c>
-      <c r="AB9" s="93" t="n"/>
-      <c r="AC9" s="108">
+      <c r="AB9" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC9" s="93" t="n"/>
+      <c r="AD9" s="108">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F9)),ISNUMBER(SEARCH("NOT APPROVED",$F9))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F9)),3,1))</f>
         <v/>
       </c>
@@ -11754,7 +12054,11 @@
           <t>Synnergie</t>
         </is>
       </c>
-      <c r="M10" s="103" t="n"/>
+      <c r="M10" s="103" t="inlineStr">
+        <is>
+          <t>Emily Fridley</t>
+        </is>
+      </c>
       <c r="N10" s="103" t="inlineStr">
         <is>
           <t>Audrey Debaere</t>
@@ -11762,30 +12066,32 @@
       </c>
       <c r="O10" s="103" t="n"/>
       <c r="P10" s="103" t="n"/>
-      <c r="Q10" s="99" t="inlineStr">
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Alex Young</t>
+        </is>
+      </c>
+      <c r="R10" s="99" t="inlineStr">
         <is>
           <t>XXL: &gt; 640 Hours</t>
         </is>
       </c>
-      <c r="R10" s="99" t="n">
+      <c r="S10" s="99" t="n">
         <v>640</v>
       </c>
-      <c r="S10" s="104">
+      <c r="T10" s="104">
         <f>$R10*65</f>
         <v/>
       </c>
-      <c r="T10" s="110" t="n">
+      <c r="U10" s="110" t="n">
         <v>0.1</v>
       </c>
-      <c r="U10" s="110" t="n">
+      <c r="V10" s="110" t="n">
         <v>0.25</v>
       </c>
-      <c r="V10" s="110" t="n">
+      <c r="W10" s="110" t="n">
         <v>0.65</v>
       </c>
-      <c r="W10" s="110" t="n">
-        <v>0</v>
-      </c>
       <c r="X10" s="110" t="n">
         <v>0</v>
       </c>
@@ -11798,12 +12104,15 @@
       <c r="AA10" s="110" t="n">
         <v>0</v>
       </c>
-      <c r="AB10" s="103" t="inlineStr">
+      <c r="AB10" s="110" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC10" s="103" t="inlineStr">
         <is>
           <t>8-9 month project</t>
         </is>
       </c>
-      <c r="AC10" s="106">
+      <c r="AD10" s="106">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F10)),ISNUMBER(SEARCH("NOT APPROVED",$F10))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F10)),3,1))</f>
         <v/>
       </c>
@@ -11855,41 +12164,47 @@
           <t>Systems Applications</t>
         </is>
       </c>
-      <c r="M11" s="93" t="n"/>
+      <c r="M11" s="93" t="inlineStr">
+        <is>
+          <t>Emily Fridley</t>
+        </is>
+      </c>
       <c r="N11" s="93" t="inlineStr">
         <is>
-          <t>Ryan Picado</t>
+          <t>Audrey Debaere</t>
         </is>
       </c>
       <c r="O11" s="93" t="n"/>
       <c r="P11" s="93" t="n"/>
-      <c r="Q11" s="89" t="inlineStr">
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Alex Young</t>
+        </is>
+      </c>
+      <c r="R11" s="89" t="inlineStr">
         <is>
           <t>S: &lt; 80 Hours</t>
         </is>
       </c>
-      <c r="R11" s="89" t="n">
+      <c r="S11" s="89" t="n">
         <v>40</v>
       </c>
-      <c r="S11" s="107">
+      <c r="T11" s="107">
         <f>$R11*65</f>
         <v/>
       </c>
-      <c r="T11" s="109" t="n">
+      <c r="U11" s="109" t="n">
         <v>0.1</v>
       </c>
-      <c r="U11" s="109" t="n">
-        <v>0</v>
-      </c>
       <c r="V11" s="109" t="n">
         <v>0</v>
       </c>
       <c r="W11" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" s="109" t="n">
         <v>0.75</v>
       </c>
-      <c r="X11" s="109" t="n">
-        <v>0</v>
-      </c>
       <c r="Y11" s="109" t="n">
         <v>0</v>
       </c>
@@ -11899,8 +12214,11 @@
       <c r="AA11" s="109" t="n">
         <v>0</v>
       </c>
-      <c r="AB11" s="93" t="n"/>
-      <c r="AC11" s="108">
+      <c r="AB11" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC11" s="93" t="n"/>
+      <c r="AD11" s="108">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F11)),ISNUMBER(SEARCH("NOT APPROVED",$F11))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F11)),3,1))</f>
         <v/>
       </c>
@@ -11952,34 +12270,44 @@
           <t>Synnergie</t>
         </is>
       </c>
-      <c r="M12" s="103" t="n"/>
-      <c r="N12" s="103" t="n"/>
+      <c r="M12" s="103" t="inlineStr">
+        <is>
+          <t>Emily Fridley</t>
+        </is>
+      </c>
+      <c r="N12" s="103" t="inlineStr">
+        <is>
+          <t>Audrey Debaere</t>
+        </is>
+      </c>
       <c r="O12" s="103" t="n"/>
       <c r="P12" s="103" t="n"/>
-      <c r="Q12" s="99" t="inlineStr">
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Alex Young</t>
+        </is>
+      </c>
+      <c r="R12" s="99" t="inlineStr">
         <is>
           <t>M: 80-160 Hours</t>
         </is>
       </c>
-      <c r="R12" s="99" t="n">
+      <c r="S12" s="99" t="n">
         <v>120</v>
       </c>
-      <c r="S12" s="104">
+      <c r="T12" s="104">
         <f>$R12*65</f>
         <v/>
       </c>
-      <c r="T12" s="110" t="n">
+      <c r="U12" s="110" t="n">
         <v>0.1</v>
       </c>
-      <c r="U12" s="110" t="n">
+      <c r="V12" s="110" t="n">
         <v>0.25</v>
       </c>
-      <c r="V12" s="110" t="n">
+      <c r="W12" s="110" t="n">
         <v>0.65</v>
       </c>
-      <c r="W12" s="110" t="n">
-        <v>0</v>
-      </c>
       <c r="X12" s="110" t="n">
         <v>0</v>
       </c>
@@ -11992,8 +12320,11 @@
       <c r="AA12" s="110" t="n">
         <v>0</v>
       </c>
-      <c r="AB12" s="103" t="n"/>
-      <c r="AC12" s="106">
+      <c r="AB12" s="110" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC12" s="103" t="n"/>
+      <c r="AD12" s="106">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F12)),ISNUMBER(SEARCH("NOT APPROVED",$F12))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F12)),3,1))</f>
         <v/>
       </c>
@@ -12045,41 +12376,47 @@
           <t>Systems Applications</t>
         </is>
       </c>
-      <c r="M13" s="93" t="n"/>
+      <c r="M13" s="93" t="inlineStr">
+        <is>
+          <t>Emily Fridley</t>
+        </is>
+      </c>
       <c r="N13" s="93" t="inlineStr">
         <is>
-          <t>Cristian Varelas</t>
+          <t>Audrey Debaere</t>
         </is>
       </c>
       <c r="O13" s="93" t="n"/>
       <c r="P13" s="93" t="n"/>
-      <c r="Q13" s="89" t="inlineStr">
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Alex Young</t>
+        </is>
+      </c>
+      <c r="R13" s="89" t="inlineStr">
         <is>
           <t>S: &lt; 80 Hours</t>
         </is>
       </c>
-      <c r="R13" s="89" t="n">
+      <c r="S13" s="89" t="n">
         <v>40</v>
       </c>
-      <c r="S13" s="107">
+      <c r="T13" s="107">
         <f>$R13*65</f>
         <v/>
       </c>
-      <c r="T13" s="109" t="n">
+      <c r="U13" s="109" t="n">
         <v>0.1</v>
       </c>
-      <c r="U13" s="109" t="n">
+      <c r="V13" s="109" t="n">
         <v>0.25</v>
       </c>
-      <c r="V13" s="109" t="n">
-        <v>0</v>
-      </c>
       <c r="W13" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="X13" s="109" t="n">
         <v>0.65</v>
       </c>
-      <c r="X13" s="109" t="n">
-        <v>0</v>
-      </c>
       <c r="Y13" s="109" t="n">
         <v>0</v>
       </c>
@@ -12089,8 +12426,11 @@
       <c r="AA13" s="109" t="n">
         <v>0</v>
       </c>
-      <c r="AB13" s="93" t="n"/>
-      <c r="AC13" s="108">
+      <c r="AB13" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC13" s="93" t="n"/>
+      <c r="AD13" s="108">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F13)),ISNUMBER(SEARCH("NOT APPROVED",$F13))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F13)),3,1))</f>
         <v/>
       </c>
@@ -12142,33 +12482,43 @@
           <t>Systems Applications</t>
         </is>
       </c>
-      <c r="M14" s="103" t="n"/>
-      <c r="N14" s="103" t="n"/>
+      <c r="M14" s="103" t="inlineStr">
+        <is>
+          <t>Emily Fridley</t>
+        </is>
+      </c>
+      <c r="N14" s="103" t="inlineStr">
+        <is>
+          <t>Audrey Debaere</t>
+        </is>
+      </c>
       <c r="O14" s="103" t="n"/>
       <c r="P14" s="103" t="n"/>
-      <c r="Q14" s="99" t="n"/>
-      <c r="R14" s="99" t="n">
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Alex Young</t>
+        </is>
+      </c>
+      <c r="R14" s="99" t="n"/>
+      <c r="S14" s="99" t="n">
         <v>200</v>
       </c>
-      <c r="S14" s="104">
+      <c r="T14" s="104">
         <f>$R14*65</f>
         <v/>
       </c>
-      <c r="T14" s="110" t="n">
+      <c r="U14" s="110" t="n">
         <v>0.1</v>
       </c>
-      <c r="U14" s="110" t="n">
-        <v>0</v>
-      </c>
       <c r="V14" s="110" t="n">
         <v>0</v>
       </c>
       <c r="W14" s="110" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" s="110" t="n">
         <v>0.75</v>
       </c>
-      <c r="X14" s="110" t="n">
-        <v>0</v>
-      </c>
       <c r="Y14" s="110" t="n">
         <v>0</v>
       </c>
@@ -12178,8 +12528,11 @@
       <c r="AA14" s="110" t="n">
         <v>0</v>
       </c>
-      <c r="AB14" s="103" t="n"/>
-      <c r="AC14" s="106">
+      <c r="AB14" s="110" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC14" s="103" t="n"/>
+      <c r="AD14" s="106">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F14)),ISNUMBER(SEARCH("NOT APPROVED",$F14))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F14)),3,1))</f>
         <v/>
       </c>
@@ -12231,33 +12584,43 @@
           <t>Systems Applications</t>
         </is>
       </c>
-      <c r="M15" s="93" t="n"/>
-      <c r="N15" s="93" t="n"/>
+      <c r="M15" s="93" t="inlineStr">
+        <is>
+          <t>Emily Fridley</t>
+        </is>
+      </c>
+      <c r="N15" s="93" t="inlineStr">
+        <is>
+          <t>Audrey Debaere</t>
+        </is>
+      </c>
       <c r="O15" s="93" t="n"/>
       <c r="P15" s="93" t="n"/>
-      <c r="Q15" s="89" t="n"/>
-      <c r="R15" s="89" t="n">
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Alex Young</t>
+        </is>
+      </c>
+      <c r="R15" s="89" t="n"/>
+      <c r="S15" s="89" t="n">
         <v>200</v>
       </c>
-      <c r="S15" s="107">
+      <c r="T15" s="107">
         <f>$R15*65</f>
         <v/>
       </c>
-      <c r="T15" s="109" t="n">
+      <c r="U15" s="109" t="n">
         <v>0.1</v>
       </c>
-      <c r="U15" s="109" t="n">
-        <v>0</v>
-      </c>
       <c r="V15" s="109" t="n">
         <v>0</v>
       </c>
       <c r="W15" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" s="109" t="n">
         <v>0.75</v>
       </c>
-      <c r="X15" s="109" t="n">
-        <v>0</v>
-      </c>
       <c r="Y15" s="109" t="n">
         <v>0</v>
       </c>
@@ -12267,8 +12630,11 @@
       <c r="AA15" s="109" t="n">
         <v>0</v>
       </c>
-      <c r="AB15" s="93" t="n"/>
-      <c r="AC15" s="108">
+      <c r="AB15" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC15" s="93" t="n"/>
+      <c r="AD15" s="108">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F15)),ISNUMBER(SEARCH("NOT APPROVED",$F15))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F15)),3,1))</f>
         <v/>
       </c>
@@ -12320,30 +12686,40 @@
           <t>Synnergie</t>
         </is>
       </c>
-      <c r="M16" s="103" t="n"/>
-      <c r="N16" s="103" t="n"/>
+      <c r="M16" s="103" t="inlineStr">
+        <is>
+          <t>Emily Fridley</t>
+        </is>
+      </c>
+      <c r="N16" s="103" t="inlineStr">
+        <is>
+          <t>Audrey Debaere</t>
+        </is>
+      </c>
       <c r="O16" s="103" t="n"/>
       <c r="P16" s="103" t="n"/>
-      <c r="Q16" s="99" t="n"/>
-      <c r="R16" s="99" t="n">
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Alex Young</t>
+        </is>
+      </c>
+      <c r="R16" s="99" t="n"/>
+      <c r="S16" s="99" t="n">
         <v>200</v>
       </c>
-      <c r="S16" s="104">
+      <c r="T16" s="104">
         <f>$R16*65</f>
         <v/>
       </c>
-      <c r="T16" s="110" t="n">
+      <c r="U16" s="110" t="n">
         <v>0.1</v>
       </c>
-      <c r="U16" s="110" t="n">
+      <c r="V16" s="110" t="n">
         <v>0.25</v>
       </c>
-      <c r="V16" s="110" t="n">
+      <c r="W16" s="110" t="n">
         <v>0.75</v>
       </c>
-      <c r="W16" s="110" t="n">
-        <v>0</v>
-      </c>
       <c r="X16" s="110" t="n">
         <v>0</v>
       </c>
@@ -12356,8 +12732,11 @@
       <c r="AA16" s="110" t="n">
         <v>0</v>
       </c>
-      <c r="AB16" s="103" t="n"/>
-      <c r="AC16" s="106">
+      <c r="AB16" s="110" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC16" s="103" t="n"/>
+      <c r="AD16" s="106">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F16)),ISNUMBER(SEARCH("NOT APPROVED",$F16))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F16)),3,1))</f>
         <v/>
       </c>
@@ -12379,19 +12758,19 @@
       <c r="N17" s="103" t="n"/>
       <c r="O17" s="103" t="n"/>
       <c r="P17" s="103" t="n"/>
-      <c r="Q17" s="99" t="n"/>
       <c r="R17" s="99" t="n"/>
-      <c r="S17" s="104" t="n"/>
-      <c r="T17" s="99" t="n"/>
+      <c r="S17" s="99" t="n"/>
+      <c r="T17" s="104" t="n"/>
       <c r="U17" s="99" t="n"/>
       <c r="V17" s="99" t="n"/>
       <c r="W17" s="99" t="n"/>
       <c r="X17" s="99" t="n"/>
       <c r="Y17" s="99" t="n"/>
-      <c r="Z17" s="105" t="n"/>
+      <c r="Z17" s="99" t="n"/>
       <c r="AA17" s="105" t="n"/>
-      <c r="AB17" s="103" t="n"/>
-      <c r="AC17" s="106">
+      <c r="AB17" s="105" t="n"/>
+      <c r="AC17" s="103" t="n"/>
+      <c r="AD17" s="106">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F17)),ISNUMBER(SEARCH("NOT APPROVED",$F17))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F17)),3,1))</f>
         <v/>
       </c>
@@ -12439,19 +12818,19 @@
       <c r="N18" s="129" t="n"/>
       <c r="O18" s="129" t="n"/>
       <c r="P18" s="129" t="n"/>
-      <c r="Q18" s="126" t="n"/>
       <c r="R18" s="126" t="n"/>
-      <c r="S18" s="130" t="n"/>
-      <c r="T18" s="126" t="n"/>
+      <c r="S18" s="126" t="n"/>
+      <c r="T18" s="130" t="n"/>
       <c r="U18" s="126" t="n"/>
       <c r="V18" s="126" t="n"/>
       <c r="W18" s="126" t="n"/>
       <c r="X18" s="126" t="n"/>
       <c r="Y18" s="126" t="n"/>
-      <c r="Z18" s="131" t="n"/>
+      <c r="Z18" s="126" t="n"/>
       <c r="AA18" s="131" t="n"/>
-      <c r="AB18" s="129" t="n"/>
-      <c r="AC18" s="132">
+      <c r="AB18" s="131" t="n"/>
+      <c r="AC18" s="129" t="n"/>
+      <c r="AD18" s="132">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F18)),ISNUMBER(SEARCH("NOT APPROVED",$F18))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F18)),3,1))</f>
         <v/>
       </c>
@@ -12499,19 +12878,19 @@
       <c r="N19" s="136" t="n"/>
       <c r="O19" s="136" t="n"/>
       <c r="P19" s="136" t="n"/>
-      <c r="Q19" s="133" t="n"/>
       <c r="R19" s="133" t="n"/>
-      <c r="S19" s="137" t="n"/>
-      <c r="T19" s="133" t="n"/>
+      <c r="S19" s="133" t="n"/>
+      <c r="T19" s="137" t="n"/>
       <c r="U19" s="133" t="n"/>
       <c r="V19" s="133" t="n"/>
       <c r="W19" s="133" t="n"/>
       <c r="X19" s="133" t="n"/>
       <c r="Y19" s="133" t="n"/>
-      <c r="Z19" s="138" t="n"/>
+      <c r="Z19" s="133" t="n"/>
       <c r="AA19" s="138" t="n"/>
-      <c r="AB19" s="136" t="n"/>
-      <c r="AC19" s="139">
+      <c r="AB19" s="138" t="n"/>
+      <c r="AC19" s="136" t="n"/>
+      <c r="AD19" s="139">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F19)),ISNUMBER(SEARCH("NOT APPROVED",$F19))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F19)),3,1))</f>
         <v/>
       </c>
@@ -12559,19 +12938,19 @@
       <c r="N20" s="122" t="n"/>
       <c r="O20" s="122" t="n"/>
       <c r="P20" s="122" t="n"/>
-      <c r="Q20" s="119" t="n"/>
       <c r="R20" s="119" t="n"/>
-      <c r="S20" s="123" t="n"/>
-      <c r="T20" s="119" t="n"/>
+      <c r="S20" s="119" t="n"/>
+      <c r="T20" s="123" t="n"/>
       <c r="U20" s="119" t="n"/>
       <c r="V20" s="119" t="n"/>
       <c r="W20" s="119" t="n"/>
       <c r="X20" s="119" t="n"/>
       <c r="Y20" s="119" t="n"/>
-      <c r="Z20" s="124" t="n"/>
+      <c r="Z20" s="119" t="n"/>
       <c r="AA20" s="124" t="n"/>
-      <c r="AB20" s="122" t="n"/>
-      <c r="AC20" s="125">
+      <c r="AB20" s="124" t="n"/>
+      <c r="AC20" s="122" t="n"/>
+      <c r="AD20" s="125">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F20)),ISNUMBER(SEARCH("NOT APPROVED",$F20))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F20)),3,1))</f>
         <v/>
       </c>
@@ -12619,19 +12998,19 @@
       <c r="N21" s="103" t="n"/>
       <c r="O21" s="103" t="n"/>
       <c r="P21" s="103" t="n"/>
-      <c r="Q21" s="99" t="n"/>
       <c r="R21" s="99" t="n"/>
-      <c r="S21" s="104" t="n"/>
-      <c r="T21" s="99" t="n"/>
+      <c r="S21" s="99" t="n"/>
+      <c r="T21" s="104" t="n"/>
       <c r="U21" s="99" t="n"/>
       <c r="V21" s="99" t="n"/>
       <c r="W21" s="99" t="n"/>
       <c r="X21" s="99" t="n"/>
       <c r="Y21" s="99" t="n"/>
-      <c r="Z21" s="105" t="n"/>
+      <c r="Z21" s="99" t="n"/>
       <c r="AA21" s="105" t="n"/>
-      <c r="AB21" s="103" t="n"/>
-      <c r="AC21" s="106">
+      <c r="AB21" s="105" t="n"/>
+      <c r="AC21" s="103" t="n"/>
+      <c r="AD21" s="106">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F21)),ISNUMBER(SEARCH("NOT APPROVED",$F21))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F21)),3,1))</f>
         <v/>
       </c>
@@ -12679,19 +13058,19 @@
       <c r="N22" s="93" t="n"/>
       <c r="O22" s="93" t="n"/>
       <c r="P22" s="93" t="n"/>
-      <c r="Q22" s="89" t="n"/>
       <c r="R22" s="89" t="n"/>
-      <c r="S22" s="107" t="n"/>
-      <c r="T22" s="89" t="n"/>
+      <c r="S22" s="89" t="n"/>
+      <c r="T22" s="107" t="n"/>
       <c r="U22" s="89" t="n"/>
       <c r="V22" s="89" t="n"/>
       <c r="W22" s="89" t="n"/>
       <c r="X22" s="89" t="n"/>
       <c r="Y22" s="89" t="n"/>
-      <c r="Z22" s="96" t="n"/>
+      <c r="Z22" s="89" t="n"/>
       <c r="AA22" s="96" t="n"/>
-      <c r="AB22" s="93" t="n"/>
-      <c r="AC22" s="108">
+      <c r="AB22" s="96" t="n"/>
+      <c r="AC22" s="93" t="n"/>
+      <c r="AD22" s="108">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F22)),ISNUMBER(SEARCH("NOT APPROVED",$F22))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F22)),3,1))</f>
         <v/>
       </c>
@@ -12739,19 +13118,19 @@
       <c r="N23" s="103" t="n"/>
       <c r="O23" s="103" t="n"/>
       <c r="P23" s="103" t="n"/>
-      <c r="Q23" s="99" t="n"/>
       <c r="R23" s="99" t="n"/>
-      <c r="S23" s="104" t="n"/>
-      <c r="T23" s="99" t="n"/>
+      <c r="S23" s="99" t="n"/>
+      <c r="T23" s="104" t="n"/>
       <c r="U23" s="99" t="n"/>
       <c r="V23" s="99" t="n"/>
       <c r="W23" s="99" t="n"/>
       <c r="X23" s="99" t="n"/>
       <c r="Y23" s="99" t="n"/>
-      <c r="Z23" s="105" t="n"/>
+      <c r="Z23" s="99" t="n"/>
       <c r="AA23" s="105" t="n"/>
-      <c r="AB23" s="103" t="n"/>
-      <c r="AC23" s="106">
+      <c r="AB23" s="105" t="n"/>
+      <c r="AC23" s="103" t="n"/>
+      <c r="AD23" s="106">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F23)),ISNUMBER(SEARCH("NOT APPROVED",$F23))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F23)),3,1))</f>
         <v/>
       </c>
@@ -12799,19 +13178,19 @@
       <c r="N24" s="93" t="n"/>
       <c r="O24" s="93" t="n"/>
       <c r="P24" s="93" t="n"/>
-      <c r="Q24" s="89" t="n"/>
       <c r="R24" s="89" t="n"/>
-      <c r="S24" s="107" t="n"/>
-      <c r="T24" s="89" t="n"/>
+      <c r="S24" s="89" t="n"/>
+      <c r="T24" s="107" t="n"/>
       <c r="U24" s="89" t="n"/>
       <c r="V24" s="89" t="n"/>
       <c r="W24" s="89" t="n"/>
       <c r="X24" s="89" t="n"/>
       <c r="Y24" s="89" t="n"/>
-      <c r="Z24" s="96" t="n"/>
+      <c r="Z24" s="89" t="n"/>
       <c r="AA24" s="96" t="n"/>
-      <c r="AB24" s="93" t="n"/>
-      <c r="AC24" s="108">
+      <c r="AB24" s="96" t="n"/>
+      <c r="AC24" s="93" t="n"/>
+      <c r="AD24" s="108">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F24)),ISNUMBER(SEARCH("NOT APPROVED",$F24))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F24)),3,1))</f>
         <v/>
       </c>
@@ -12859,19 +13238,19 @@
       <c r="N25" s="103" t="n"/>
       <c r="O25" s="103" t="n"/>
       <c r="P25" s="103" t="n"/>
-      <c r="Q25" s="99" t="n"/>
       <c r="R25" s="99" t="n"/>
-      <c r="S25" s="104" t="n"/>
-      <c r="T25" s="99" t="n"/>
+      <c r="S25" s="99" t="n"/>
+      <c r="T25" s="104" t="n"/>
       <c r="U25" s="99" t="n"/>
       <c r="V25" s="99" t="n"/>
       <c r="W25" s="99" t="n"/>
       <c r="X25" s="99" t="n"/>
       <c r="Y25" s="99" t="n"/>
-      <c r="Z25" s="105" t="n"/>
+      <c r="Z25" s="99" t="n"/>
       <c r="AA25" s="105" t="n"/>
-      <c r="AB25" s="103" t="n"/>
-      <c r="AC25" s="106">
+      <c r="AB25" s="105" t="n"/>
+      <c r="AC25" s="103" t="n"/>
+      <c r="AD25" s="106">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F25)),ISNUMBER(SEARCH("NOT APPROVED",$F25))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F25)),3,1))</f>
         <v/>
       </c>
@@ -12931,25 +13310,25 @@
       </c>
       <c r="O26" s="93" t="n"/>
       <c r="P26" s="93" t="n"/>
-      <c r="Q26" s="89" t="inlineStr">
+      <c r="R26" s="89" t="inlineStr">
         <is>
           <t>M: 80-160 Hours</t>
         </is>
       </c>
-      <c r="R26" s="89" t="n">
+      <c r="S26" s="89" t="n">
         <v>120</v>
       </c>
-      <c r="S26" s="107" t="n"/>
-      <c r="T26" s="89" t="n"/>
+      <c r="T26" s="107" t="n"/>
       <c r="U26" s="89" t="n"/>
       <c r="V26" s="89" t="n"/>
       <c r="W26" s="89" t="n"/>
       <c r="X26" s="89" t="n"/>
       <c r="Y26" s="89" t="n"/>
-      <c r="Z26" s="96" t="n"/>
+      <c r="Z26" s="89" t="n"/>
       <c r="AA26" s="96" t="n"/>
-      <c r="AB26" s="93" t="n"/>
-      <c r="AC26" s="108">
+      <c r="AB26" s="96" t="n"/>
+      <c r="AC26" s="93" t="n"/>
+      <c r="AD26" s="108">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F26)),ISNUMBER(SEARCH("NOT APPROVED",$F26))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F26)),3,1))</f>
         <v/>
       </c>
@@ -13021,34 +13400,34 @@
           <t>Sangamesh Koti</t>
         </is>
       </c>
-      <c r="Q27" s="99" t="inlineStr">
+      <c r="R27" s="99" t="inlineStr">
         <is>
           <t>M: 80-160 Hours</t>
         </is>
       </c>
-      <c r="R27" s="99" t="n">
+      <c r="S27" s="99" t="n">
         <v>120</v>
       </c>
-      <c r="S27" s="104">
+      <c r="T27" s="104">
         <f>$R27*65</f>
         <v/>
       </c>
-      <c r="T27" s="105" t="n">
+      <c r="U27" s="105" t="n">
         <v>0.1</v>
       </c>
-      <c r="U27" s="105" t="n">
+      <c r="V27" s="105" t="n">
         <v>0.25</v>
       </c>
-      <c r="V27" s="105" t="n">
+      <c r="W27" s="105" t="n">
         <v>0.75</v>
       </c>
-      <c r="W27" s="105" t="n"/>
       <c r="X27" s="105" t="n"/>
       <c r="Y27" s="105" t="n"/>
       <c r="Z27" s="105" t="n"/>
       <c r="AA27" s="105" t="n"/>
-      <c r="AB27" s="103" t="n"/>
-      <c r="AC27" s="106">
+      <c r="AB27" s="105" t="n"/>
+      <c r="AC27" s="103" t="n"/>
+      <c r="AD27" s="106">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F27)),ISNUMBER(SEARCH("NOT APPROVED",$F27))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F27)),3,1))</f>
         <v/>
       </c>
@@ -13112,34 +13491,34 @@
       </c>
       <c r="O28" s="103" t="n"/>
       <c r="P28" s="103" t="n"/>
-      <c r="Q28" s="99" t="inlineStr">
+      <c r="R28" s="99" t="inlineStr">
         <is>
           <t>M: 80-160 Hours</t>
         </is>
       </c>
-      <c r="R28" s="99" t="n">
+      <c r="S28" s="99" t="n">
         <v>120</v>
       </c>
-      <c r="S28" s="104">
+      <c r="T28" s="104">
         <f>$R28*65</f>
         <v/>
       </c>
-      <c r="T28" s="105" t="n">
+      <c r="U28" s="105" t="n">
         <v>0.1</v>
       </c>
-      <c r="U28" s="105" t="n">
+      <c r="V28" s="105" t="n">
         <v>0.25</v>
       </c>
-      <c r="V28" s="105" t="n">
+      <c r="W28" s="105" t="n">
         <v>0.65</v>
       </c>
-      <c r="W28" s="105" t="n"/>
       <c r="X28" s="105" t="n"/>
       <c r="Y28" s="105" t="n"/>
       <c r="Z28" s="105" t="n"/>
       <c r="AA28" s="105" t="n"/>
-      <c r="AB28" s="103" t="n"/>
-      <c r="AC28" s="106">
+      <c r="AB28" s="105" t="n"/>
+      <c r="AC28" s="103" t="n"/>
+      <c r="AD28" s="106">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F28)),ISNUMBER(SEARCH("NOT APPROVED",$F28))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F28)),3,1))</f>
         <v/>
       </c>
@@ -13203,28 +13582,28 @@
           <t>Michael House</t>
         </is>
       </c>
-      <c r="Q29" s="99" t="n"/>
-      <c r="R29" s="99" t="n">
+      <c r="R29" s="99" t="n"/>
+      <c r="S29" s="99" t="n">
         <v>120</v>
       </c>
-      <c r="S29" s="104">
+      <c r="T29" s="104">
         <f>$R29*65</f>
         <v/>
       </c>
-      <c r="T29" s="105" t="n">
+      <c r="U29" s="105" t="n">
         <v>0.1</v>
       </c>
-      <c r="U29" s="105" t="n"/>
       <c r="V29" s="105" t="n"/>
       <c r="W29" s="105" t="n"/>
-      <c r="X29" s="105" t="n">
+      <c r="X29" s="105" t="n"/>
+      <c r="Y29" s="105" t="n">
         <v>0.5</v>
       </c>
-      <c r="Y29" s="105" t="n"/>
       <c r="Z29" s="105" t="n"/>
       <c r="AA29" s="105" t="n"/>
-      <c r="AB29" s="103" t="n"/>
-      <c r="AC29" s="106">
+      <c r="AB29" s="105" t="n"/>
+      <c r="AC29" s="103" t="n"/>
+      <c r="AD29" s="106">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F29)),ISNUMBER(SEARCH("NOT APPROVED",$F29))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F29)),3,1))</f>
         <v/>
       </c>
@@ -13294,27 +13673,27 @@
           <t>Jonathon Gonzalez</t>
         </is>
       </c>
-      <c r="Q30" s="99" t="inlineStr">
+      <c r="R30" s="99" t="inlineStr">
         <is>
           <t>S: &lt; 80 Hours</t>
         </is>
       </c>
-      <c r="R30" s="99" t="n">
+      <c r="S30" s="99" t="n">
         <v>60</v>
       </c>
-      <c r="S30" s="104" t="n">
+      <c r="T30" s="104" t="n">
         <v>11895</v>
       </c>
-      <c r="T30" s="99" t="n"/>
       <c r="U30" s="99" t="n"/>
       <c r="V30" s="99" t="n"/>
       <c r="W30" s="99" t="n"/>
       <c r="X30" s="99" t="n"/>
       <c r="Y30" s="99" t="n"/>
-      <c r="Z30" s="105" t="n"/>
+      <c r="Z30" s="99" t="n"/>
       <c r="AA30" s="105" t="n"/>
-      <c r="AB30" s="103" t="n"/>
-      <c r="AC30" s="106">
+      <c r="AB30" s="105" t="n"/>
+      <c r="AC30" s="103" t="n"/>
+      <c r="AD30" s="106">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F30)),ISNUMBER(SEARCH("NOT APPROVED",$F30))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F30)),3,1))</f>
         <v/>
       </c>
@@ -13384,27 +13763,27 @@
           <t>Ravindra Reddy</t>
         </is>
       </c>
-      <c r="Q31" s="89" t="inlineStr">
+      <c r="R31" s="89" t="inlineStr">
         <is>
           <t>L: 160-320 Hours</t>
         </is>
       </c>
-      <c r="R31" s="89" t="n">
+      <c r="S31" s="89" t="n">
         <v>360</v>
       </c>
-      <c r="S31" s="107" t="n">
+      <c r="T31" s="107" t="n">
         <v>16120</v>
       </c>
-      <c r="T31" s="89" t="n"/>
       <c r="U31" s="89" t="n"/>
       <c r="V31" s="89" t="n"/>
       <c r="W31" s="89" t="n"/>
       <c r="X31" s="89" t="n"/>
       <c r="Y31" s="89" t="n"/>
-      <c r="Z31" s="96" t="n"/>
+      <c r="Z31" s="89" t="n"/>
       <c r="AA31" s="96" t="n"/>
-      <c r="AB31" s="93" t="n"/>
-      <c r="AC31" s="108">
+      <c r="AB31" s="96" t="n"/>
+      <c r="AC31" s="93" t="n"/>
+      <c r="AD31" s="108">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F31)),ISNUMBER(SEARCH("NOT APPROVED",$F31))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F31)),3,1))</f>
         <v/>
       </c>
@@ -13474,27 +13853,27 @@
           <t>Bhavya Reddy</t>
         </is>
       </c>
-      <c r="Q32" s="99" t="inlineStr">
+      <c r="R32" s="99" t="inlineStr">
         <is>
           <t>L: 160-320 Hours</t>
         </is>
       </c>
-      <c r="R32" s="99" t="n">
+      <c r="S32" s="99" t="n">
         <v>310</v>
       </c>
-      <c r="S32" s="104" t="n">
+      <c r="T32" s="104" t="n">
         <v>1625</v>
       </c>
-      <c r="T32" s="99" t="n"/>
       <c r="U32" s="99" t="n"/>
       <c r="V32" s="99" t="n"/>
       <c r="W32" s="99" t="n"/>
       <c r="X32" s="99" t="n"/>
       <c r="Y32" s="99" t="n"/>
-      <c r="Z32" s="105" t="n"/>
+      <c r="Z32" s="99" t="n"/>
       <c r="AA32" s="105" t="n"/>
-      <c r="AB32" s="103" t="n"/>
-      <c r="AC32" s="106">
+      <c r="AB32" s="105" t="n"/>
+      <c r="AC32" s="103" t="n"/>
+      <c r="AD32" s="106">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F32)),ISNUMBER(SEARCH("NOT APPROVED",$F32))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F32)),3,1))</f>
         <v/>
       </c>
@@ -13564,27 +13943,27 @@
           <t>Sangamesh Koti</t>
         </is>
       </c>
-      <c r="Q33" s="89" t="inlineStr">
+      <c r="R33" s="89" t="inlineStr">
         <is>
           <t>M: 80-160 Hours</t>
         </is>
       </c>
-      <c r="R33" s="89" t="n">
+      <c r="S33" s="89" t="n">
         <v>160</v>
       </c>
-      <c r="S33" s="107" t="n">
+      <c r="T33" s="107" t="n">
         <v>260</v>
       </c>
-      <c r="T33" s="89" t="n"/>
       <c r="U33" s="89" t="n"/>
       <c r="V33" s="89" t="n"/>
       <c r="W33" s="89" t="n"/>
       <c r="X33" s="89" t="n"/>
       <c r="Y33" s="89" t="n"/>
-      <c r="Z33" s="96" t="n"/>
+      <c r="Z33" s="89" t="n"/>
       <c r="AA33" s="96" t="n"/>
-      <c r="AB33" s="93" t="n"/>
-      <c r="AC33" s="108">
+      <c r="AB33" s="96" t="n"/>
+      <c r="AC33" s="93" t="n"/>
+      <c r="AD33" s="108">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F33)),ISNUMBER(SEARCH("NOT APPROVED",$F33))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F33)),3,1))</f>
         <v/>
       </c>
@@ -13654,29 +14033,29 @@
           <t>Vishnu Premen</t>
         </is>
       </c>
-      <c r="Q34" s="99" t="inlineStr">
+      <c r="R34" s="99" t="inlineStr">
         <is>
           <t>M: 80-160 Hours</t>
         </is>
       </c>
-      <c r="R34" s="99" t="n">
+      <c r="S34" s="99" t="n">
         <v>120</v>
       </c>
-      <c r="S34" s="104" t="n"/>
-      <c r="T34" s="99" t="n"/>
+      <c r="T34" s="104" t="n"/>
       <c r="U34" s="99" t="n"/>
       <c r="V34" s="99" t="n"/>
       <c r="W34" s="99" t="n"/>
       <c r="X34" s="99" t="n"/>
       <c r="Y34" s="99" t="n"/>
-      <c r="Z34" s="105" t="n"/>
+      <c r="Z34" s="99" t="n"/>
       <c r="AA34" s="105" t="n"/>
-      <c r="AB34" s="103" t="inlineStr">
+      <c r="AB34" s="105" t="n"/>
+      <c r="AC34" s="103" t="inlineStr">
         <is>
           <t>NAPA not ready</t>
         </is>
       </c>
-      <c r="AC34" s="106">
+      <c r="AD34" s="106">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F34)),ISNUMBER(SEARCH("NOT APPROVED",$F34))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F34)),3,1))</f>
         <v/>
       </c>
@@ -13742,21 +14121,21 @@
           <t>Justin Senour</t>
         </is>
       </c>
-      <c r="Q35" s="89" t="n"/>
-      <c r="R35" s="89" t="n">
-        <v>0</v>
-      </c>
-      <c r="S35" s="107" t="n"/>
-      <c r="T35" s="89" t="n"/>
+      <c r="R35" s="89" t="n"/>
+      <c r="S35" s="89" t="n">
+        <v>0</v>
+      </c>
+      <c r="T35" s="107" t="n"/>
       <c r="U35" s="89" t="n"/>
       <c r="V35" s="89" t="n"/>
       <c r="W35" s="89" t="n"/>
       <c r="X35" s="89" t="n"/>
       <c r="Y35" s="89" t="n"/>
-      <c r="Z35" s="96" t="n"/>
+      <c r="Z35" s="89" t="n"/>
       <c r="AA35" s="96" t="n"/>
-      <c r="AB35" s="93" t="n"/>
-      <c r="AC35" s="108">
+      <c r="AB35" s="96" t="n"/>
+      <c r="AC35" s="93" t="n"/>
+      <c r="AD35" s="108">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F35)),ISNUMBER(SEARCH("NOT APPROVED",$F35))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F35)),3,1))</f>
         <v/>
       </c>
@@ -13822,21 +14201,21 @@
           <t>Michael House</t>
         </is>
       </c>
-      <c r="Q36" s="99" t="n"/>
-      <c r="R36" s="99" t="n">
-        <v>0</v>
-      </c>
-      <c r="S36" s="104" t="n"/>
-      <c r="T36" s="99" t="n"/>
+      <c r="R36" s="99" t="n"/>
+      <c r="S36" s="99" t="n">
+        <v>0</v>
+      </c>
+      <c r="T36" s="104" t="n"/>
       <c r="U36" s="99" t="n"/>
       <c r="V36" s="99" t="n"/>
       <c r="W36" s="99" t="n"/>
       <c r="X36" s="99" t="n"/>
       <c r="Y36" s="99" t="n"/>
-      <c r="Z36" s="105" t="n"/>
+      <c r="Z36" s="99" t="n"/>
       <c r="AA36" s="105" t="n"/>
-      <c r="AB36" s="103" t="n"/>
-      <c r="AC36" s="106">
+      <c r="AB36" s="105" t="n"/>
+      <c r="AC36" s="103" t="n"/>
+      <c r="AD36" s="106">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F36)),ISNUMBER(SEARCH("NOT APPROVED",$F36))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F36)),3,1))</f>
         <v/>
       </c>
@@ -13892,25 +14271,25 @@
       <c r="N37" s="93" t="n"/>
       <c r="O37" s="93" t="n"/>
       <c r="P37" s="93" t="n"/>
-      <c r="Q37" s="89" t="inlineStr">
+      <c r="R37" s="89" t="inlineStr">
         <is>
           <t>S: &lt; 80 Hours</t>
         </is>
       </c>
-      <c r="R37" s="89" t="n">
+      <c r="S37" s="89" t="n">
         <v>40</v>
       </c>
-      <c r="S37" s="107" t="n"/>
-      <c r="T37" s="89" t="n"/>
+      <c r="T37" s="107" t="n"/>
       <c r="U37" s="89" t="n"/>
       <c r="V37" s="89" t="n"/>
       <c r="W37" s="89" t="n"/>
       <c r="X37" s="89" t="n"/>
       <c r="Y37" s="89" t="n"/>
-      <c r="Z37" s="96" t="n"/>
+      <c r="Z37" s="89" t="n"/>
       <c r="AA37" s="96" t="n"/>
-      <c r="AB37" s="93" t="n"/>
-      <c r="AC37" s="108">
+      <c r="AB37" s="96" t="n"/>
+      <c r="AC37" s="93" t="n"/>
+      <c r="AD37" s="108">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F37)),ISNUMBER(SEARCH("NOT APPROVED",$F37))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F37)),3,1))</f>
         <v/>
       </c>
@@ -13980,21 +14359,21 @@
           <t>Sangamesh Koti</t>
         </is>
       </c>
-      <c r="Q38" s="99" t="n"/>
-      <c r="R38" s="99" t="n">
+      <c r="R38" s="99" t="n"/>
+      <c r="S38" s="99" t="n">
         <v>320</v>
       </c>
-      <c r="S38" s="104" t="n"/>
-      <c r="T38" s="99" t="n"/>
+      <c r="T38" s="104" t="n"/>
       <c r="U38" s="99" t="n"/>
       <c r="V38" s="99" t="n"/>
       <c r="W38" s="99" t="n"/>
       <c r="X38" s="99" t="n"/>
       <c r="Y38" s="99" t="n"/>
-      <c r="Z38" s="105" t="n"/>
+      <c r="Z38" s="99" t="n"/>
       <c r="AA38" s="105" t="n"/>
-      <c r="AB38" s="103" t="n"/>
-      <c r="AC38" s="106">
+      <c r="AB38" s="105" t="n"/>
+      <c r="AC38" s="103" t="n"/>
+      <c r="AD38" s="106">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F38)),ISNUMBER(SEARCH("NOT APPROVED",$F38))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F38)),3,1))</f>
         <v/>
       </c>
@@ -14054,25 +14433,25 @@
       </c>
       <c r="O39" s="93" t="n"/>
       <c r="P39" s="93" t="n"/>
-      <c r="Q39" s="89" t="inlineStr">
+      <c r="R39" s="89" t="inlineStr">
         <is>
           <t>S: &lt; 80 Hours</t>
         </is>
       </c>
-      <c r="R39" s="89" t="n">
+      <c r="S39" s="89" t="n">
         <v>40</v>
       </c>
-      <c r="S39" s="107" t="n"/>
-      <c r="T39" s="89" t="n"/>
+      <c r="T39" s="107" t="n"/>
       <c r="U39" s="89" t="n"/>
       <c r="V39" s="89" t="n"/>
       <c r="W39" s="89" t="n"/>
       <c r="X39" s="89" t="n"/>
       <c r="Y39" s="89" t="n"/>
-      <c r="Z39" s="96" t="n"/>
+      <c r="Z39" s="89" t="n"/>
       <c r="AA39" s="96" t="n"/>
-      <c r="AB39" s="93" t="n"/>
-      <c r="AC39" s="108">
+      <c r="AB39" s="96" t="n"/>
+      <c r="AC39" s="93" t="n"/>
+      <c r="AD39" s="108">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F39)),ISNUMBER(SEARCH("NOT APPROVED",$F39))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F39)),3,1))</f>
         <v/>
       </c>
@@ -14124,7 +14503,11 @@
           <t>Synnergie</t>
         </is>
       </c>
-      <c r="M40" s="103" t="n"/>
+      <c r="M40" s="103" t="inlineStr">
+        <is>
+          <t>Emily Fridley</t>
+        </is>
+      </c>
       <c r="N40" s="103" t="inlineStr">
         <is>
           <t>Audrey Debaere</t>
@@ -14132,25 +14515,30 @@
       </c>
       <c r="O40" s="103" t="n"/>
       <c r="P40" s="103" t="n"/>
-      <c r="Q40" s="99" t="inlineStr">
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Alex Young</t>
+        </is>
+      </c>
+      <c r="R40" s="99" t="inlineStr">
         <is>
           <t>S: &lt; 80 Hours</t>
         </is>
       </c>
-      <c r="R40" s="99" t="n">
+      <c r="S40" s="99" t="n">
         <v>80</v>
       </c>
-      <c r="S40" s="104" t="n"/>
-      <c r="T40" s="99" t="n"/>
+      <c r="T40" s="104" t="n"/>
       <c r="U40" s="99" t="n"/>
       <c r="V40" s="99" t="n"/>
       <c r="W40" s="99" t="n"/>
       <c r="X40" s="99" t="n"/>
       <c r="Y40" s="99" t="n"/>
-      <c r="Z40" s="105" t="n"/>
+      <c r="Z40" s="99" t="n"/>
       <c r="AA40" s="105" t="n"/>
-      <c r="AB40" s="103" t="n"/>
-      <c r="AC40" s="106">
+      <c r="AB40" s="105" t="n"/>
+      <c r="AC40" s="103" t="n"/>
+      <c r="AD40" s="106">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F40)),ISNUMBER(SEARCH("NOT APPROVED",$F40))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F40)),3,1))</f>
         <v/>
       </c>
@@ -14210,25 +14598,25 @@
       </c>
       <c r="O41" s="93" t="n"/>
       <c r="P41" s="93" t="n"/>
-      <c r="Q41" s="89" t="inlineStr">
+      <c r="R41" s="89" t="inlineStr">
         <is>
           <t>L: 160-320 Hours</t>
         </is>
       </c>
-      <c r="R41" s="89" t="n">
+      <c r="S41" s="89" t="n">
         <v>320</v>
       </c>
-      <c r="S41" s="107" t="n"/>
-      <c r="T41" s="89" t="n"/>
+      <c r="T41" s="107" t="n"/>
       <c r="U41" s="89" t="n"/>
       <c r="V41" s="89" t="n"/>
       <c r="W41" s="89" t="n"/>
       <c r="X41" s="89" t="n"/>
       <c r="Y41" s="89" t="n"/>
-      <c r="Z41" s="96" t="n"/>
+      <c r="Z41" s="89" t="n"/>
       <c r="AA41" s="96" t="n"/>
-      <c r="AB41" s="93" t="n"/>
-      <c r="AC41" s="108">
+      <c r="AB41" s="96" t="n"/>
+      <c r="AC41" s="93" t="n"/>
+      <c r="AD41" s="108">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F41)),ISNUMBER(SEARCH("NOT APPROVED",$F41))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F41)),3,1))</f>
         <v/>
       </c>
@@ -14284,10 +14672,14 @@
           <t>Systems Applications</t>
         </is>
       </c>
-      <c r="M42" s="114" t="n"/>
+      <c r="M42" s="114" t="inlineStr">
+        <is>
+          <t>Emily Fridley</t>
+        </is>
+      </c>
       <c r="N42" s="114" t="inlineStr">
         <is>
-          <t>Jim Young</t>
+          <t>Audrey Debaere</t>
         </is>
       </c>
       <c r="O42" s="114" t="n"/>
@@ -14296,25 +14688,30 @@
           <t>Alex Young</t>
         </is>
       </c>
-      <c r="Q42" s="111" t="inlineStr">
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Alex Young</t>
+        </is>
+      </c>
+      <c r="R42" s="111" t="inlineStr">
         <is>
           <t>S: &lt; 80 Hours</t>
         </is>
       </c>
-      <c r="R42" s="111" t="n">
+      <c r="S42" s="111" t="n">
         <v>40</v>
       </c>
-      <c r="S42" s="115" t="n"/>
-      <c r="T42" s="111" t="n"/>
+      <c r="T42" s="115" t="n"/>
       <c r="U42" s="111" t="n"/>
       <c r="V42" s="111" t="n"/>
       <c r="W42" s="111" t="n"/>
       <c r="X42" s="111" t="n"/>
       <c r="Y42" s="111" t="n"/>
-      <c r="Z42" s="116" t="n"/>
+      <c r="Z42" s="111" t="n"/>
       <c r="AA42" s="116" t="n"/>
-      <c r="AB42" s="114" t="n"/>
-      <c r="AC42" s="118">
+      <c r="AB42" s="116" t="n"/>
+      <c r="AC42" s="114" t="n"/>
+      <c r="AD42" s="118">
         <f>IF(OR(ISNUMBER(SEARCH("POSTPONED",$F42)),ISNUMBER(SEARCH("NOT APPROVED",$F42))),2,IF(ISNUMBER(SEARCH("COMPLETE",$F42)),3,1))</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Rebuild app as Streamlit executive dashboard with 7-page navigation
Replace chat-only UI with a full visual dashboard: Executive Summary,
Portfolio, Project Detail (with scheduling availability engine),
Project Editor (form-based Excel write-back), Capacity, Timeline/Gantt,
and AI Assistant. Adds cached data layer, reusable components, cross-page
navigation, and test data across all active projects.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ETE PMO Resource Planner.xlsx
+++ b/ETE PMO Resource Planner.xlsx
@@ -8751,9 +8751,7 @@
       <c r="E23" s="304" t="n">
         <v>220</v>
       </c>
-      <c r="F23" s="282" t="n">
-        <v/>
-      </c>
+      <c r="F23" s="282" t="n"/>
       <c r="G23" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -8792,9 +8790,7 @@
       <c r="E24" s="282" t="n">
         <v>40</v>
       </c>
-      <c r="F24" s="282" t="n">
-        <v/>
-      </c>
+      <c r="F24" s="282" t="n"/>
       <c r="G24" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -8833,9 +8829,7 @@
       <c r="E25" s="304" t="n">
         <v>170</v>
       </c>
-      <c r="F25" s="282" t="n">
-        <v/>
-      </c>
+      <c r="F25" s="282" t="n"/>
       <c r="G25" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -8874,9 +8868,7 @@
       <c r="E26" s="304" t="n">
         <v>544</v>
       </c>
-      <c r="F26" s="282" t="n">
-        <v/>
-      </c>
+      <c r="F26" s="282" t="n"/>
       <c r="G26" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -8915,9 +8907,7 @@
       <c r="E27" s="282" t="n">
         <v>120</v>
       </c>
-      <c r="F27" s="282" t="n">
-        <v/>
-      </c>
+      <c r="F27" s="282" t="n"/>
       <c r="G27" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -8956,9 +8946,7 @@
       <c r="E28" s="304" t="n">
         <v>148</v>
       </c>
-      <c r="F28" s="282" t="n">
-        <v/>
-      </c>
+      <c r="F28" s="282" t="n"/>
       <c r="G28" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -8997,9 +8985,7 @@
       <c r="E29" s="304" t="n">
         <v>84</v>
       </c>
-      <c r="F29" s="282" t="n">
-        <v/>
-      </c>
+      <c r="F29" s="282" t="n"/>
       <c r="G29" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -9038,9 +9024,7 @@
       <c r="E30" s="304" t="n">
         <v>170</v>
       </c>
-      <c r="F30" s="282" t="n">
-        <v/>
-      </c>
+      <c r="F30" s="282" t="n"/>
       <c r="G30" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -9079,9 +9063,7 @@
       <c r="E31" s="304" t="n">
         <v>204</v>
       </c>
-      <c r="F31" s="282" t="n">
-        <v/>
-      </c>
+      <c r="F31" s="282" t="n"/>
       <c r="G31" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -9120,9 +9102,7 @@
       <c r="E32" s="282" t="n">
         <v>640</v>
       </c>
-      <c r="F32" s="282" t="n">
-        <v/>
-      </c>
+      <c r="F32" s="282" t="n"/>
       <c r="G32" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -9161,9 +9141,7 @@
       <c r="E33" s="282" t="n">
         <v>120</v>
       </c>
-      <c r="F33" s="282" t="n">
-        <v/>
-      </c>
+      <c r="F33" s="282" t="n"/>
       <c r="G33" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -9202,9 +9180,7 @@
       <c r="E34" s="304" t="n">
         <v>34</v>
       </c>
-      <c r="F34" s="282" t="n">
-        <v/>
-      </c>
+      <c r="F34" s="282" t="n"/>
       <c r="G34" s="282" t="inlineStr">
         <is>
           <t>IT Business Analyst/SME</t>
@@ -10017,33 +9993,15 @@
       <c r="C22" s="282" t="n">
         <v>200</v>
       </c>
-      <c r="D22" s="282" t="n">
-        <v/>
-      </c>
-      <c r="E22" s="290" t="n">
-        <v/>
-      </c>
-      <c r="F22" s="290" t="n">
-        <v/>
-      </c>
-      <c r="G22" s="290" t="n">
-        <v/>
-      </c>
-      <c r="H22" s="290" t="n">
-        <v/>
-      </c>
-      <c r="I22" s="290" t="n">
-        <v/>
-      </c>
-      <c r="J22" s="290" t="n">
-        <v/>
-      </c>
-      <c r="K22" s="290" t="n">
-        <v/>
-      </c>
-      <c r="L22" s="290" t="n">
-        <v/>
-      </c>
+      <c r="D22" s="282" t="n"/>
+      <c r="E22" s="290" t="n"/>
+      <c r="F22" s="290" t="n"/>
+      <c r="G22" s="290" t="n"/>
+      <c r="H22" s="290" t="n"/>
+      <c r="I22" s="290" t="n"/>
+      <c r="J22" s="290" t="n"/>
+      <c r="K22" s="290" t="n"/>
+      <c r="L22" s="290" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="287" t="inlineStr">
@@ -10059,33 +10017,15 @@
       <c r="C23" s="282" t="n">
         <v>40</v>
       </c>
-      <c r="D23" s="282" t="n">
-        <v/>
-      </c>
-      <c r="E23" s="290" t="n">
-        <v/>
-      </c>
-      <c r="F23" s="290" t="n">
-        <v/>
-      </c>
-      <c r="G23" s="290" t="n">
-        <v/>
-      </c>
-      <c r="H23" s="290" t="n">
-        <v/>
-      </c>
-      <c r="I23" s="290" t="n">
-        <v/>
-      </c>
-      <c r="J23" s="290" t="n">
-        <v/>
-      </c>
-      <c r="K23" s="290" t="n">
-        <v/>
-      </c>
-      <c r="L23" s="290" t="n">
-        <v/>
-      </c>
+      <c r="D23" s="282" t="n"/>
+      <c r="E23" s="290" t="n"/>
+      <c r="F23" s="290" t="n"/>
+      <c r="G23" s="290" t="n"/>
+      <c r="H23" s="290" t="n"/>
+      <c r="I23" s="290" t="n"/>
+      <c r="J23" s="290" t="n"/>
+      <c r="K23" s="290" t="n"/>
+      <c r="L23" s="290" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="287" t="inlineStr">
@@ -10101,33 +10041,15 @@
       <c r="C24" s="282" t="n">
         <v>200</v>
       </c>
-      <c r="D24" s="282" t="n">
-        <v/>
-      </c>
-      <c r="E24" s="290" t="n">
-        <v/>
-      </c>
-      <c r="F24" s="290" t="n">
-        <v/>
-      </c>
-      <c r="G24" s="290" t="n">
-        <v/>
-      </c>
-      <c r="H24" s="290" t="n">
-        <v/>
-      </c>
-      <c r="I24" s="290" t="n">
-        <v/>
-      </c>
-      <c r="J24" s="290" t="n">
-        <v/>
-      </c>
-      <c r="K24" s="290" t="n">
-        <v/>
-      </c>
-      <c r="L24" s="290" t="n">
-        <v/>
-      </c>
+      <c r="D24" s="282" t="n"/>
+      <c r="E24" s="290" t="n"/>
+      <c r="F24" s="290" t="n"/>
+      <c r="G24" s="290" t="n"/>
+      <c r="H24" s="290" t="n"/>
+      <c r="I24" s="290" t="n"/>
+      <c r="J24" s="290" t="n"/>
+      <c r="K24" s="290" t="n"/>
+      <c r="L24" s="290" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="287" t="inlineStr">
@@ -10143,33 +10065,15 @@
       <c r="C25" s="282" t="n">
         <v>640</v>
       </c>
-      <c r="D25" s="282" t="n">
-        <v/>
-      </c>
-      <c r="E25" s="290" t="n">
-        <v/>
-      </c>
-      <c r="F25" s="290" t="n">
-        <v/>
-      </c>
-      <c r="G25" s="290" t="n">
-        <v/>
-      </c>
-      <c r="H25" s="290" t="n">
-        <v/>
-      </c>
-      <c r="I25" s="290" t="n">
-        <v/>
-      </c>
-      <c r="J25" s="290" t="n">
-        <v/>
-      </c>
-      <c r="K25" s="290" t="n">
-        <v/>
-      </c>
-      <c r="L25" s="290" t="n">
-        <v/>
-      </c>
+      <c r="D25" s="282" t="n"/>
+      <c r="E25" s="290" t="n"/>
+      <c r="F25" s="290" t="n"/>
+      <c r="G25" s="290" t="n"/>
+      <c r="H25" s="290" t="n"/>
+      <c r="I25" s="290" t="n"/>
+      <c r="J25" s="290" t="n"/>
+      <c r="K25" s="290" t="n"/>
+      <c r="L25" s="290" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="287" t="inlineStr">
@@ -10185,33 +10089,15 @@
       <c r="C26" s="282" t="n">
         <v>120</v>
       </c>
-      <c r="D26" s="282" t="n">
-        <v/>
-      </c>
-      <c r="E26" s="290" t="n">
-        <v/>
-      </c>
-      <c r="F26" s="290" t="n">
-        <v/>
-      </c>
-      <c r="G26" s="290" t="n">
-        <v/>
-      </c>
-      <c r="H26" s="290" t="n">
-        <v/>
-      </c>
-      <c r="I26" s="290" t="n">
-        <v/>
-      </c>
-      <c r="J26" s="290" t="n">
-        <v/>
-      </c>
-      <c r="K26" s="290" t="n">
-        <v/>
-      </c>
-      <c r="L26" s="290" t="n">
-        <v/>
-      </c>
+      <c r="D26" s="282" t="n"/>
+      <c r="E26" s="290" t="n"/>
+      <c r="F26" s="290" t="n"/>
+      <c r="G26" s="290" t="n"/>
+      <c r="H26" s="290" t="n"/>
+      <c r="I26" s="290" t="n"/>
+      <c r="J26" s="290" t="n"/>
+      <c r="K26" s="290" t="n"/>
+      <c r="L26" s="290" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="287" t="inlineStr">
@@ -10227,33 +10113,15 @@
       <c r="C27" s="282" t="n">
         <v>1480</v>
       </c>
-      <c r="D27" s="282" t="n">
-        <v/>
-      </c>
-      <c r="E27" s="290" t="n">
-        <v/>
-      </c>
-      <c r="F27" s="290" t="n">
-        <v/>
-      </c>
-      <c r="G27" s="290" t="n">
-        <v/>
-      </c>
-      <c r="H27" s="290" t="n">
-        <v/>
-      </c>
-      <c r="I27" s="290" t="n">
-        <v/>
-      </c>
-      <c r="J27" s="290" t="n">
-        <v/>
-      </c>
-      <c r="K27" s="290" t="n">
-        <v/>
-      </c>
-      <c r="L27" s="290" t="n">
-        <v/>
-      </c>
+      <c r="D27" s="282" t="n"/>
+      <c r="E27" s="290" t="n"/>
+      <c r="F27" s="290" t="n"/>
+      <c r="G27" s="290" t="n"/>
+      <c r="H27" s="290" t="n"/>
+      <c r="I27" s="290" t="n"/>
+      <c r="J27" s="290" t="n"/>
+      <c r="K27" s="290" t="n"/>
+      <c r="L27" s="290" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="287" t="inlineStr">
@@ -10269,33 +10137,15 @@
       <c r="C28" s="282" t="n">
         <v>240</v>
       </c>
-      <c r="D28" s="282" t="n">
-        <v/>
-      </c>
-      <c r="E28" s="290" t="n">
-        <v/>
-      </c>
-      <c r="F28" s="290" t="n">
-        <v/>
-      </c>
-      <c r="G28" s="290" t="n">
-        <v/>
-      </c>
-      <c r="H28" s="290" t="n">
-        <v/>
-      </c>
-      <c r="I28" s="290" t="n">
-        <v/>
-      </c>
-      <c r="J28" s="290" t="n">
-        <v/>
-      </c>
-      <c r="K28" s="290" t="n">
-        <v/>
-      </c>
-      <c r="L28" s="290" t="n">
-        <v/>
-      </c>
+      <c r="D28" s="282" t="n"/>
+      <c r="E28" s="290" t="n"/>
+      <c r="F28" s="290" t="n"/>
+      <c r="G28" s="290" t="n"/>
+      <c r="H28" s="290" t="n"/>
+      <c r="I28" s="290" t="n"/>
+      <c r="J28" s="290" t="n"/>
+      <c r="K28" s="290" t="n"/>
+      <c r="L28" s="290" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="287" t="inlineStr">
@@ -10311,33 +10161,15 @@
       <c r="C29" s="282" t="n">
         <v>200</v>
       </c>
-      <c r="D29" s="282" t="n">
-        <v/>
-      </c>
-      <c r="E29" s="290" t="n">
-        <v/>
-      </c>
-      <c r="F29" s="290" t="n">
-        <v/>
-      </c>
-      <c r="G29" s="290" t="n">
-        <v/>
-      </c>
-      <c r="H29" s="290" t="n">
-        <v/>
-      </c>
-      <c r="I29" s="290" t="n">
-        <v/>
-      </c>
-      <c r="J29" s="290" t="n">
-        <v/>
-      </c>
-      <c r="K29" s="290" t="n">
-        <v/>
-      </c>
-      <c r="L29" s="290" t="n">
-        <v/>
-      </c>
+      <c r="D29" s="282" t="n"/>
+      <c r="E29" s="290" t="n"/>
+      <c r="F29" s="290" t="n"/>
+      <c r="G29" s="290" t="n"/>
+      <c r="H29" s="290" t="n"/>
+      <c r="I29" s="290" t="n"/>
+      <c r="J29" s="290" t="n"/>
+      <c r="K29" s="290" t="n"/>
+      <c r="L29" s="290" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="287" t="inlineStr">
@@ -10353,33 +10185,15 @@
       <c r="C30" s="282" t="n">
         <v>240</v>
       </c>
-      <c r="D30" s="282" t="n">
-        <v/>
-      </c>
-      <c r="E30" s="290" t="n">
-        <v/>
-      </c>
-      <c r="F30" s="290" t="n">
-        <v/>
-      </c>
-      <c r="G30" s="290" t="n">
-        <v/>
-      </c>
-      <c r="H30" s="290" t="n">
-        <v/>
-      </c>
-      <c r="I30" s="290" t="n">
-        <v/>
-      </c>
-      <c r="J30" s="290" t="n">
-        <v/>
-      </c>
-      <c r="K30" s="290" t="n">
-        <v/>
-      </c>
-      <c r="L30" s="290" t="n">
-        <v/>
-      </c>
+      <c r="D30" s="282" t="n"/>
+      <c r="E30" s="290" t="n"/>
+      <c r="F30" s="290" t="n"/>
+      <c r="G30" s="290" t="n"/>
+      <c r="H30" s="290" t="n"/>
+      <c r="I30" s="290" t="n"/>
+      <c r="J30" s="290" t="n"/>
+      <c r="K30" s="290" t="n"/>
+      <c r="L30" s="290" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="287" t="inlineStr">
@@ -10395,33 +10209,15 @@
       <c r="C31" s="282" t="n">
         <v>640</v>
       </c>
-      <c r="D31" s="282" t="n">
-        <v/>
-      </c>
-      <c r="E31" s="290" t="n">
-        <v/>
-      </c>
-      <c r="F31" s="290" t="n">
-        <v/>
-      </c>
-      <c r="G31" s="290" t="n">
-        <v/>
-      </c>
-      <c r="H31" s="290" t="n">
-        <v/>
-      </c>
-      <c r="I31" s="290" t="n">
-        <v/>
-      </c>
-      <c r="J31" s="290" t="n">
-        <v/>
-      </c>
-      <c r="K31" s="290" t="n">
-        <v/>
-      </c>
-      <c r="L31" s="290" t="n">
-        <v/>
-      </c>
+      <c r="D31" s="282" t="n"/>
+      <c r="E31" s="290" t="n"/>
+      <c r="F31" s="290" t="n"/>
+      <c r="G31" s="290" t="n"/>
+      <c r="H31" s="290" t="n"/>
+      <c r="I31" s="290" t="n"/>
+      <c r="J31" s="290" t="n"/>
+      <c r="K31" s="290" t="n"/>
+      <c r="L31" s="290" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="287" t="inlineStr">
@@ -10437,33 +10233,15 @@
       <c r="C32" s="282" t="n">
         <v>120</v>
       </c>
-      <c r="D32" s="282" t="n">
-        <v/>
-      </c>
-      <c r="E32" s="290" t="n">
-        <v/>
-      </c>
-      <c r="F32" s="290" t="n">
-        <v/>
-      </c>
-      <c r="G32" s="290" t="n">
-        <v/>
-      </c>
-      <c r="H32" s="290" t="n">
-        <v/>
-      </c>
-      <c r="I32" s="290" t="n">
-        <v/>
-      </c>
-      <c r="J32" s="290" t="n">
-        <v/>
-      </c>
-      <c r="K32" s="290" t="n">
-        <v/>
-      </c>
-      <c r="L32" s="290" t="n">
-        <v/>
-      </c>
+      <c r="D32" s="282" t="n"/>
+      <c r="E32" s="290" t="n"/>
+      <c r="F32" s="290" t="n"/>
+      <c r="G32" s="290" t="n"/>
+      <c r="H32" s="290" t="n"/>
+      <c r="I32" s="290" t="n"/>
+      <c r="J32" s="290" t="n"/>
+      <c r="K32" s="290" t="n"/>
+      <c r="L32" s="290" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="287" t="inlineStr">
@@ -10479,33 +10257,15 @@
       <c r="C33" s="282" t="n">
         <v>40</v>
       </c>
-      <c r="D33" s="282" t="n">
-        <v/>
-      </c>
-      <c r="E33" s="290" t="n">
-        <v/>
-      </c>
-      <c r="F33" s="290" t="n">
-        <v/>
-      </c>
-      <c r="G33" s="290" t="n">
-        <v/>
-      </c>
-      <c r="H33" s="290" t="n">
-        <v/>
-      </c>
-      <c r="I33" s="290" t="n">
-        <v/>
-      </c>
-      <c r="J33" s="290" t="n">
-        <v/>
-      </c>
-      <c r="K33" s="290" t="n">
-        <v/>
-      </c>
-      <c r="L33" s="290" t="n">
-        <v/>
-      </c>
+      <c r="D33" s="282" t="n"/>
+      <c r="E33" s="290" t="n"/>
+      <c r="F33" s="290" t="n"/>
+      <c r="G33" s="290" t="n"/>
+      <c r="H33" s="290" t="n"/>
+      <c r="I33" s="290" t="n"/>
+      <c r="J33" s="290" t="n"/>
+      <c r="K33" s="290" t="n"/>
+      <c r="L33" s="290" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="273" t="inlineStr">
@@ -11429,7 +11189,7 @@
       </c>
       <c r="F4" s="89" t="inlineStr">
         <is>
-          <t>📋 NEEDS TECHNICAL SPEC</t>
+          <t>NEEDS TECHNICAL SPEC</t>
         </is>
       </c>
       <c r="G4" s="91" t="n">
@@ -11462,8 +11222,16 @@
           <t>Audrey Debaere</t>
         </is>
       </c>
-      <c r="O4" s="93" t="n"/>
-      <c r="P4" s="93" t="n"/>
+      <c r="O4" s="93" t="inlineStr">
+        <is>
+          <t>Deepak Gudwani</t>
+        </is>
+      </c>
+      <c r="P4" s="93" t="inlineStr">
+        <is>
+          <t>Bhavya Reddy</t>
+        </is>
+      </c>
       <c r="Q4" t="inlineStr">
         <is>
           <t>Alex Young</t>
@@ -11484,13 +11252,27 @@
       <c r="U4" s="95" t="n">
         <v>0.1</v>
       </c>
-      <c r="V4" s="95" t="n"/>
-      <c r="W4" s="95" t="n"/>
-      <c r="X4" s="95" t="n"/>
-      <c r="Y4" s="95" t="n"/>
-      <c r="Z4" s="95" t="n"/>
-      <c r="AA4" s="96" t="n"/>
-      <c r="AB4" s="96" t="n"/>
+      <c r="V4" s="95" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W4" s="95" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="X4" s="95" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Y4" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="95" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AA4" s="96" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="AB4" s="96" t="n">
+        <v>0</v>
+      </c>
       <c r="AC4" s="97" t="inlineStr">
         <is>
           <t>Completed Q1</t>
@@ -11562,8 +11344,16 @@
           <t>Audrey Debaere</t>
         </is>
       </c>
-      <c r="O5" s="103" t="n"/>
-      <c r="P5" s="103" t="n"/>
+      <c r="O5" s="103" t="inlineStr">
+        <is>
+          <t>Ajay Kumar</t>
+        </is>
+      </c>
+      <c r="P5" s="103" t="inlineStr">
+        <is>
+          <t>Sangamesh Koti</t>
+        </is>
+      </c>
       <c r="Q5" t="inlineStr">
         <is>
           <t>Alex Young</t>
@@ -11584,9 +11374,15 @@
       <c r="U5" s="105" t="n">
         <v>0.1</v>
       </c>
-      <c r="V5" s="105" t="n"/>
-      <c r="W5" s="105" t="n"/>
-      <c r="X5" s="105" t="n"/>
+      <c r="V5" s="105" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W5" s="105" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="X5" s="105" t="n">
+        <v>0.75</v>
+      </c>
       <c r="Y5" s="105" t="n"/>
       <c r="Z5" s="105" t="n"/>
       <c r="AA5" s="105" t="n">
@@ -11660,7 +11456,11 @@
           <t>Audrey Debaere</t>
         </is>
       </c>
-      <c r="O6" s="93" t="n"/>
+      <c r="O6" s="93" t="inlineStr">
+        <is>
+          <t>Ajay Kumar</t>
+        </is>
+      </c>
       <c r="P6" s="93" t="inlineStr">
         <is>
           <t>Colin Olson</t>
@@ -11686,14 +11486,20 @@
       <c r="U6" s="96" t="n">
         <v>0.1</v>
       </c>
-      <c r="V6" s="96" t="n"/>
-      <c r="W6" s="96" t="n"/>
+      <c r="V6" s="96" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W6" s="96" t="n">
+        <v>0.25</v>
+      </c>
       <c r="X6" s="96" t="n">
         <v>0.75</v>
       </c>
       <c r="Y6" s="96" t="n"/>
       <c r="Z6" s="96" t="n"/>
-      <c r="AA6" s="96" t="n"/>
+      <c r="AA6" s="96" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AB6" s="96" t="n"/>
       <c r="AC6" s="93" t="n"/>
       <c r="AD6" s="108">
@@ -11762,8 +11568,16 @@
           <t>Audrey Debaere</t>
         </is>
       </c>
-      <c r="O7" s="93" t="n"/>
-      <c r="P7" s="93" t="n"/>
+      <c r="O7" s="93" t="inlineStr">
+        <is>
+          <t>Deepak Gudwani</t>
+        </is>
+      </c>
+      <c r="P7" s="93" t="inlineStr">
+        <is>
+          <t>Sarath Yeturu</t>
+        </is>
+      </c>
       <c r="Q7" t="inlineStr">
         <is>
           <t>Alex Young</t>
@@ -11771,7 +11585,7 @@
       </c>
       <c r="R7" s="89" t="n"/>
       <c r="S7" s="89" t="n">
-        <v>0</v>
+        <v>320</v>
       </c>
       <c r="T7" s="107">
         <f>$R7*65</f>
@@ -11780,12 +11594,20 @@
       <c r="U7" s="96" t="n">
         <v>0.1</v>
       </c>
-      <c r="V7" s="96" t="n"/>
-      <c r="W7" s="96" t="n"/>
-      <c r="X7" s="96" t="n"/>
+      <c r="V7" s="96" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W7" s="96" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="X7" s="96" t="n">
+        <v>0.5</v>
+      </c>
       <c r="Y7" s="96" t="n"/>
       <c r="Z7" s="96" t="n"/>
-      <c r="AA7" s="96" t="n"/>
+      <c r="AA7" s="96" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AB7" s="96" t="n"/>
       <c r="AC7" s="93" t="n"/>
       <c r="AD7" s="108">
@@ -11890,10 +11712,16 @@
       <c r="W8" s="96" t="n">
         <v>0.65</v>
       </c>
-      <c r="X8" s="96" t="n"/>
+      <c r="X8" s="96" t="n">
+        <v>0.75</v>
+      </c>
       <c r="Y8" s="96" t="n"/>
-      <c r="Z8" s="96" t="n"/>
-      <c r="AA8" s="96" t="n"/>
+      <c r="Z8" s="96" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AA8" s="96" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AB8" s="96" t="n"/>
       <c r="AC8" s="93" t="n"/>
       <c r="AD8" s="108">
@@ -11940,8 +11768,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="I9" s="314" t="n"/>
-      <c r="J9" s="314" t="n"/>
+      <c r="I9" s="314" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J9" s="314" t="n">
+        <v>46281</v>
+      </c>
       <c r="K9" s="314" t="n"/>
       <c r="L9" s="89" t="inlineStr">
         <is>
@@ -11958,8 +11790,16 @@
           <t>Audrey Debaere</t>
         </is>
       </c>
-      <c r="O9" s="93" t="n"/>
-      <c r="P9" s="93" t="n"/>
+      <c r="O9" s="93" t="inlineStr">
+        <is>
+          <t>Ajay Kumar</t>
+        </is>
+      </c>
+      <c r="P9" s="93" t="inlineStr">
+        <is>
+          <t>Sarath Yeturu</t>
+        </is>
+      </c>
       <c r="Q9" t="inlineStr">
         <is>
           <t>Alex Young</t>
@@ -11981,22 +11821,22 @@
         <v>0.1</v>
       </c>
       <c r="V9" s="109" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="W9" s="109" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="X9" s="109" t="n">
         <v>0.75</v>
       </c>
       <c r="Y9" s="109" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="Z9" s="109" t="n">
         <v>0</v>
       </c>
       <c r="AA9" s="109" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AB9" s="109" t="n">
         <v>0</v>
@@ -12046,8 +11886,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="I10" s="315" t="n"/>
-      <c r="J10" s="315" t="n"/>
+      <c r="I10" s="315" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J10" s="315" t="n">
+        <v>46162</v>
+      </c>
       <c r="K10" s="315" t="n"/>
       <c r="L10" s="99" t="inlineStr">
         <is>
@@ -12064,8 +11908,16 @@
           <t>Audrey Debaere</t>
         </is>
       </c>
-      <c r="O10" s="103" t="n"/>
-      <c r="P10" s="103" t="n"/>
+      <c r="O10" s="103" t="inlineStr">
+        <is>
+          <t>Ajay Kumar</t>
+        </is>
+      </c>
+      <c r="P10" s="103" t="inlineStr">
+        <is>
+          <t>Bhavya Reddy</t>
+        </is>
+      </c>
       <c r="Q10" t="inlineStr">
         <is>
           <t>Alex Young</t>
@@ -12087,13 +11939,13 @@
         <v>0.1</v>
       </c>
       <c r="V10" s="110" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W10" s="110" t="n">
         <v>0.25</v>
       </c>
-      <c r="W10" s="110" t="n">
-        <v>0.65</v>
-      </c>
       <c r="X10" s="110" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="Y10" s="110" t="n">
         <v>0</v>
@@ -12102,7 +11954,7 @@
         <v>0</v>
       </c>
       <c r="AA10" s="110" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AB10" s="110" t="n">
         <v>0</v>
@@ -12156,8 +12008,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="I11" s="314" t="n"/>
-      <c r="J11" s="314" t="n"/>
+      <c r="I11" s="314" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J11" s="314" t="n">
+        <v>46141</v>
+      </c>
       <c r="K11" s="314" t="n"/>
       <c r="L11" s="89" t="inlineStr">
         <is>
@@ -12174,8 +12030,16 @@
           <t>Audrey Debaere</t>
         </is>
       </c>
-      <c r="O11" s="93" t="n"/>
-      <c r="P11" s="93" t="n"/>
+      <c r="O11" s="93" t="inlineStr">
+        <is>
+          <t>Ajay Kumar</t>
+        </is>
+      </c>
+      <c r="P11" s="93" t="inlineStr">
+        <is>
+          <t>Bhavya Reddy</t>
+        </is>
+      </c>
       <c r="Q11" t="inlineStr">
         <is>
           <t>Alex Young</t>
@@ -12197,22 +12061,22 @@
         <v>0.1</v>
       </c>
       <c r="V11" s="109" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="W11" s="109" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="X11" s="109" t="n">
         <v>0.75</v>
       </c>
       <c r="Y11" s="109" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="Z11" s="109" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="AA11" s="109" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AB11" s="109" t="n">
         <v>0</v>
@@ -12262,8 +12126,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="I12" s="315" t="n"/>
-      <c r="J12" s="315" t="n"/>
+      <c r="I12" s="315" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J12" s="315" t="n">
+        <v>46197</v>
+      </c>
       <c r="K12" s="315" t="n"/>
       <c r="L12" s="99" t="inlineStr">
         <is>
@@ -12280,8 +12148,16 @@
           <t>Audrey Debaere</t>
         </is>
       </c>
-      <c r="O12" s="103" t="n"/>
-      <c r="P12" s="103" t="n"/>
+      <c r="O12" s="103" t="inlineStr">
+        <is>
+          <t>Deepak Gudwani</t>
+        </is>
+      </c>
+      <c r="P12" s="103" t="inlineStr">
+        <is>
+          <t>Ravindra Reddy</t>
+        </is>
+      </c>
       <c r="Q12" t="inlineStr">
         <is>
           <t>Alex Young</t>
@@ -12303,22 +12179,22 @@
         <v>0.1</v>
       </c>
       <c r="V12" s="110" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W12" s="110" t="n">
         <v>0.25</v>
       </c>
-      <c r="W12" s="110" t="n">
-        <v>0.65</v>
-      </c>
       <c r="X12" s="110" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="Y12" s="110" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="Z12" s="110" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AA12" s="110" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AB12" s="110" t="n">
         <v>0</v>
@@ -12368,8 +12244,12 @@
           <t>Highest</t>
         </is>
       </c>
-      <c r="I13" s="314" t="n"/>
-      <c r="J13" s="314" t="n"/>
+      <c r="I13" s="314" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J13" s="314" t="n">
+        <v>46190</v>
+      </c>
       <c r="K13" s="314" t="n"/>
       <c r="L13" s="89" t="inlineStr">
         <is>
@@ -12386,8 +12266,16 @@
           <t>Audrey Debaere</t>
         </is>
       </c>
-      <c r="O13" s="93" t="n"/>
-      <c r="P13" s="93" t="n"/>
+      <c r="O13" s="93" t="inlineStr">
+        <is>
+          <t>Ajay Kumar</t>
+        </is>
+      </c>
+      <c r="P13" s="93" t="inlineStr">
+        <is>
+          <t>Sarath Yeturu</t>
+        </is>
+      </c>
       <c r="Q13" t="inlineStr">
         <is>
           <t>Alex Young</t>
@@ -12409,10 +12297,10 @@
         <v>0.1</v>
       </c>
       <c r="V13" s="109" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W13" s="109" t="n">
         <v>0.25</v>
-      </c>
-      <c r="W13" s="109" t="n">
-        <v>0</v>
       </c>
       <c r="X13" s="109" t="n">
         <v>0.65</v>
@@ -12421,10 +12309,10 @@
         <v>0</v>
       </c>
       <c r="Z13" s="109" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="AA13" s="109" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AB13" s="109" t="n">
         <v>0</v>
@@ -12474,8 +12362,12 @@
           <t>Highest</t>
         </is>
       </c>
-      <c r="I14" s="315" t="n"/>
-      <c r="J14" s="315" t="n"/>
+      <c r="I14" s="315" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J14" s="315" t="n">
+        <v>46190</v>
+      </c>
       <c r="K14" s="315" t="n"/>
       <c r="L14" s="99" t="inlineStr">
         <is>
@@ -12492,8 +12384,16 @@
           <t>Audrey Debaere</t>
         </is>
       </c>
-      <c r="O14" s="103" t="n"/>
-      <c r="P14" s="103" t="n"/>
+      <c r="O14" s="103" t="inlineStr">
+        <is>
+          <t>Ajay Kumar</t>
+        </is>
+      </c>
+      <c r="P14" s="103" t="inlineStr">
+        <is>
+          <t>Bhavya Reddy</t>
+        </is>
+      </c>
       <c r="Q14" t="inlineStr">
         <is>
           <t>Alex Young</t>
@@ -12511,10 +12411,10 @@
         <v>0.1</v>
       </c>
       <c r="V14" s="110" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="W14" s="110" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="X14" s="110" t="n">
         <v>0.75</v>
@@ -12526,7 +12426,7 @@
         <v>0</v>
       </c>
       <c r="AA14" s="110" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AB14" s="110" t="n">
         <v>0</v>
@@ -12576,8 +12476,12 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="I15" s="314" t="n"/>
-      <c r="J15" s="314" t="n"/>
+      <c r="I15" s="314" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J15" s="314" t="n">
+        <v>46169</v>
+      </c>
       <c r="K15" s="314" t="n"/>
       <c r="L15" s="89" t="inlineStr">
         <is>
@@ -12594,8 +12498,16 @@
           <t>Audrey Debaere</t>
         </is>
       </c>
-      <c r="O15" s="93" t="n"/>
-      <c r="P15" s="93" t="n"/>
+      <c r="O15" s="93" t="inlineStr">
+        <is>
+          <t>Deepak Gudwani</t>
+        </is>
+      </c>
+      <c r="P15" s="93" t="inlineStr">
+        <is>
+          <t>Ravindra Reddy</t>
+        </is>
+      </c>
       <c r="Q15" t="inlineStr">
         <is>
           <t>Alex Young</t>
@@ -12613,22 +12525,22 @@
         <v>0.1</v>
       </c>
       <c r="V15" s="109" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="W15" s="109" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="X15" s="109" t="n">
         <v>0.75</v>
       </c>
       <c r="Y15" s="109" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="Z15" s="109" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AA15" s="109" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AB15" s="109" t="n">
         <v>0</v>
@@ -12678,8 +12590,12 @@
           <t>Highest</t>
         </is>
       </c>
-      <c r="I16" s="315" t="n"/>
-      <c r="J16" s="315" t="n"/>
+      <c r="I16" s="315" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J16" s="315" t="n">
+        <v>46162</v>
+      </c>
       <c r="K16" s="315" t="n"/>
       <c r="L16" s="99" t="inlineStr">
         <is>
@@ -12696,8 +12612,16 @@
           <t>Audrey Debaere</t>
         </is>
       </c>
-      <c r="O16" s="103" t="n"/>
-      <c r="P16" s="103" t="n"/>
+      <c r="O16" s="103" t="inlineStr">
+        <is>
+          <t>Ajay Kumar</t>
+        </is>
+      </c>
+      <c r="P16" s="103" t="inlineStr">
+        <is>
+          <t>Sarath Yeturu</t>
+        </is>
+      </c>
       <c r="Q16" t="inlineStr">
         <is>
           <t>Alex Young</t>
@@ -12715,22 +12639,22 @@
         <v>0.1</v>
       </c>
       <c r="V16" s="110" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W16" s="110" t="n">
         <v>0.25</v>
       </c>
-      <c r="W16" s="110" t="n">
+      <c r="X16" s="110" t="n">
         <v>0.75</v>
       </c>
-      <c r="X16" s="110" t="n">
-        <v>0</v>
-      </c>
       <c r="Y16" s="110" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="Z16" s="110" t="n">
         <v>0</v>
       </c>
       <c r="AA16" s="110" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AB16" s="110" t="n">
         <v>0</v>
@@ -12810,8 +12734,12 @@
         <v>0</v>
       </c>
       <c r="H18" s="126" t="n"/>
-      <c r="I18" s="316" t="n"/>
-      <c r="J18" s="316" t="n"/>
+      <c r="I18" s="316" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J18" s="316" t="n">
+        <v>46288</v>
+      </c>
       <c r="K18" s="316" t="n"/>
       <c r="L18" s="126" t="n"/>
       <c r="M18" s="129" t="n"/>
@@ -12870,8 +12798,12 @@
         <v>0</v>
       </c>
       <c r="H19" s="133" t="n"/>
-      <c r="I19" s="317" t="n"/>
-      <c r="J19" s="317" t="n"/>
+      <c r="I19" s="317" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J19" s="317" t="n">
+        <v>46260</v>
+      </c>
       <c r="K19" s="317" t="n"/>
       <c r="L19" s="133" t="n"/>
       <c r="M19" s="136" t="n"/>
@@ -12930,8 +12862,12 @@
         <v>0</v>
       </c>
       <c r="H20" s="119" t="n"/>
-      <c r="I20" s="318" t="n"/>
-      <c r="J20" s="318" t="n"/>
+      <c r="I20" s="318" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J20" s="318" t="n">
+        <v>46155</v>
+      </c>
       <c r="K20" s="318" t="n"/>
       <c r="L20" s="119" t="n"/>
       <c r="M20" s="122" t="n"/>
@@ -12990,8 +12926,12 @@
         <v>0</v>
       </c>
       <c r="H21" s="99" t="n"/>
-      <c r="I21" s="315" t="n"/>
-      <c r="J21" s="315" t="n"/>
+      <c r="I21" s="315" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J21" s="315" t="n">
+        <v>46267</v>
+      </c>
       <c r="K21" s="315" t="n"/>
       <c r="L21" s="99" t="n"/>
       <c r="M21" s="103" t="n"/>
@@ -13050,8 +12990,12 @@
         <v>0</v>
       </c>
       <c r="H22" s="89" t="n"/>
-      <c r="I22" s="314" t="n"/>
-      <c r="J22" s="314" t="n"/>
+      <c r="I22" s="314" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J22" s="314" t="n">
+        <v>46232</v>
+      </c>
       <c r="K22" s="314" t="n"/>
       <c r="L22" s="89" t="n"/>
       <c r="M22" s="93" t="n"/>
@@ -13110,8 +13054,12 @@
         <v>0</v>
       </c>
       <c r="H23" s="99" t="n"/>
-      <c r="I23" s="315" t="n"/>
-      <c r="J23" s="315" t="n"/>
+      <c r="I23" s="315" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J23" s="315" t="n">
+        <v>46148</v>
+      </c>
       <c r="K23" s="315" t="n"/>
       <c r="L23" s="99" t="n"/>
       <c r="M23" s="103" t="n"/>
@@ -13170,8 +13118,12 @@
         <v>0</v>
       </c>
       <c r="H24" s="89" t="n"/>
-      <c r="I24" s="314" t="n"/>
-      <c r="J24" s="314" t="n"/>
+      <c r="I24" s="314" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J24" s="314" t="n">
+        <v>46141</v>
+      </c>
       <c r="K24" s="314" t="n"/>
       <c r="L24" s="89" t="n"/>
       <c r="M24" s="93" t="n"/>
@@ -13230,8 +13182,12 @@
         <v>0</v>
       </c>
       <c r="H25" s="99" t="n"/>
-      <c r="I25" s="315" t="n"/>
-      <c r="J25" s="315" t="n"/>
+      <c r="I25" s="315" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J25" s="315" t="n">
+        <v>46155</v>
+      </c>
       <c r="K25" s="315" t="n"/>
       <c r="L25" s="99" t="n"/>
       <c r="M25" s="103" t="n"/>
@@ -13294,22 +13250,38 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I26" s="314" t="n"/>
-      <c r="J26" s="314" t="n"/>
+      <c r="I26" s="314" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J26" s="314" t="n">
+        <v>46183</v>
+      </c>
       <c r="K26" s="314" t="n"/>
       <c r="L26" s="89" t="inlineStr">
         <is>
           <t>Systems Applications</t>
         </is>
       </c>
-      <c r="M26" s="93" t="n"/>
+      <c r="M26" s="93" t="inlineStr">
+        <is>
+          <t>Brett Anderson</t>
+        </is>
+      </c>
       <c r="N26" s="93" t="inlineStr">
         <is>
           <t>Jim Young</t>
         </is>
       </c>
-      <c r="O26" s="93" t="n"/>
-      <c r="P26" s="93" t="n"/>
+      <c r="O26" s="93" t="inlineStr">
+        <is>
+          <t>Deepak Gudwani</t>
+        </is>
+      </c>
+      <c r="P26" s="93" t="inlineStr">
+        <is>
+          <t>Sarath Yeturu</t>
+        </is>
+      </c>
       <c r="R26" s="89" t="inlineStr">
         <is>
           <t>M: 80-160 Hours</t>
@@ -13319,13 +13291,25 @@
         <v>120</v>
       </c>
       <c r="T26" s="107" t="n"/>
-      <c r="U26" s="89" t="n"/>
-      <c r="V26" s="89" t="n"/>
-      <c r="W26" s="89" t="n"/>
-      <c r="X26" s="89" t="n"/>
+      <c r="U26" s="89" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="V26" s="89" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W26" s="89" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="X26" s="89" t="n">
+        <v>0.75</v>
+      </c>
       <c r="Y26" s="89" t="n"/>
-      <c r="Z26" s="89" t="n"/>
-      <c r="AA26" s="96" t="n"/>
+      <c r="Z26" s="89" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AA26" s="96" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AB26" s="96" t="n"/>
       <c r="AC26" s="93" t="n"/>
       <c r="AD26" s="108">
@@ -13384,7 +13368,11 @@
           <t>Synnergie</t>
         </is>
       </c>
-      <c r="M27" s="103" t="n"/>
+      <c r="M27" s="103" t="inlineStr">
+        <is>
+          <t>Emily Fridley</t>
+        </is>
+      </c>
       <c r="N27" s="103" t="inlineStr">
         <is>
           <t>Audrey Debaere</t>
@@ -13421,10 +13409,14 @@
       <c r="W27" s="105" t="n">
         <v>0.75</v>
       </c>
-      <c r="X27" s="105" t="n"/>
+      <c r="X27" s="105" t="n">
+        <v>0.5</v>
+      </c>
       <c r="Y27" s="105" t="n"/>
       <c r="Z27" s="105" t="n"/>
-      <c r="AA27" s="105" t="n"/>
+      <c r="AA27" s="105" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AB27" s="105" t="n"/>
       <c r="AC27" s="103" t="n"/>
       <c r="AD27" s="106">
@@ -13483,14 +13475,26 @@
           <t>Synnergie</t>
         </is>
       </c>
-      <c r="M28" s="103" t="n"/>
+      <c r="M28" s="103" t="inlineStr">
+        <is>
+          <t>Bettina Kotico</t>
+        </is>
+      </c>
       <c r="N28" s="103" t="inlineStr">
         <is>
           <t>Audrey Debaere</t>
         </is>
       </c>
-      <c r="O28" s="103" t="n"/>
-      <c r="P28" s="103" t="n"/>
+      <c r="O28" s="103" t="inlineStr">
+        <is>
+          <t>Ajay Kumar</t>
+        </is>
+      </c>
+      <c r="P28" s="103" t="inlineStr">
+        <is>
+          <t>Sarath Yeturu</t>
+        </is>
+      </c>
       <c r="R28" s="99" t="inlineStr">
         <is>
           <t>M: 80-160 Hours</t>
@@ -13507,15 +13511,23 @@
         <v>0.1</v>
       </c>
       <c r="V28" s="105" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W28" s="105" t="n">
         <v>0.25</v>
       </c>
-      <c r="W28" s="105" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="X28" s="105" t="n"/>
-      <c r="Y28" s="105" t="n"/>
-      <c r="Z28" s="105" t="n"/>
-      <c r="AA28" s="105" t="n"/>
+      <c r="X28" s="105" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="Y28" s="105" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Z28" s="105" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AA28" s="105" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AB28" s="105" t="n"/>
       <c r="AC28" s="103" t="n"/>
       <c r="AD28" s="106">
@@ -13574,9 +13586,21 @@
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="M29" s="103" t="n"/>
-      <c r="N29" s="103" t="n"/>
-      <c r="O29" s="103" t="n"/>
+      <c r="M29" s="103" t="inlineStr">
+        <is>
+          <t>Emily Fridley</t>
+        </is>
+      </c>
+      <c r="N29" s="103" t="inlineStr">
+        <is>
+          <t>Ryan Picado</t>
+        </is>
+      </c>
+      <c r="O29" s="103" t="inlineStr">
+        <is>
+          <t>Ajay Kumar</t>
+        </is>
+      </c>
       <c r="P29" s="103" t="inlineStr">
         <is>
           <t>Michael House</t>
@@ -13591,16 +13615,24 @@
         <v/>
       </c>
       <c r="U29" s="105" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="V29" s="105" t="n"/>
-      <c r="W29" s="105" t="n"/>
-      <c r="X29" s="105" t="n"/>
+        <v>0.15</v>
+      </c>
+      <c r="V29" s="105" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W29" s="105" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="X29" s="105" t="n">
+        <v>0.5</v>
+      </c>
       <c r="Y29" s="105" t="n">
         <v>0.5</v>
       </c>
       <c r="Z29" s="105" t="n"/>
-      <c r="AA29" s="105" t="n"/>
+      <c r="AA29" s="105" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AB29" s="105" t="n"/>
       <c r="AC29" s="103" t="n"/>
       <c r="AD29" s="106">
@@ -13661,13 +13693,21 @@
           <t>Systems Applications</t>
         </is>
       </c>
-      <c r="M30" s="103" t="n"/>
+      <c r="M30" s="103" t="inlineStr">
+        <is>
+          <t>Brett Anderson</t>
+        </is>
+      </c>
       <c r="N30" s="103" t="inlineStr">
         <is>
           <t>Jim Young</t>
         </is>
       </c>
-      <c r="O30" s="103" t="n"/>
+      <c r="O30" s="103" t="inlineStr">
+        <is>
+          <t>Deepak Gudwani</t>
+        </is>
+      </c>
       <c r="P30" s="103" t="inlineStr">
         <is>
           <t>Jonathon Gonzalez</t>
@@ -13684,13 +13724,25 @@
       <c r="T30" s="104" t="n">
         <v>11895</v>
       </c>
-      <c r="U30" s="99" t="n"/>
-      <c r="V30" s="99" t="n"/>
-      <c r="W30" s="99" t="n"/>
-      <c r="X30" s="99" t="n"/>
+      <c r="U30" s="99" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="V30" s="99" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W30" s="99" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="X30" s="99" t="n">
+        <v>0.5</v>
+      </c>
       <c r="Y30" s="99" t="n"/>
-      <c r="Z30" s="99" t="n"/>
-      <c r="AA30" s="105" t="n"/>
+      <c r="Z30" s="99" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AA30" s="105" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AB30" s="105" t="n"/>
       <c r="AC30" s="103" t="n"/>
       <c r="AD30" s="106">
@@ -13751,13 +13803,21 @@
           <t>Synnergie</t>
         </is>
       </c>
-      <c r="M31" s="93" t="n"/>
+      <c r="M31" s="93" t="inlineStr">
+        <is>
+          <t>Emily Fridley</t>
+        </is>
+      </c>
       <c r="N31" s="93" t="inlineStr">
         <is>
           <t>Audrey Debaere</t>
         </is>
       </c>
-      <c r="O31" s="93" t="n"/>
+      <c r="O31" s="93" t="inlineStr">
+        <is>
+          <t>Ajay Kumar</t>
+        </is>
+      </c>
       <c r="P31" s="93" t="inlineStr">
         <is>
           <t>Ravindra Reddy</t>
@@ -13774,13 +13834,25 @@
       <c r="T31" s="107" t="n">
         <v>16120</v>
       </c>
-      <c r="U31" s="89" t="n"/>
-      <c r="V31" s="89" t="n"/>
-      <c r="W31" s="89" t="n"/>
-      <c r="X31" s="89" t="n"/>
-      <c r="Y31" s="89" t="n"/>
+      <c r="U31" s="89" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="V31" s="89" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W31" s="89" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="X31" s="89" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="Y31" s="89" t="n">
+        <v>0.1</v>
+      </c>
       <c r="Z31" s="89" t="n"/>
-      <c r="AA31" s="96" t="n"/>
+      <c r="AA31" s="96" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AB31" s="96" t="n"/>
       <c r="AC31" s="93" t="n"/>
       <c r="AD31" s="108">
@@ -13841,13 +13913,21 @@
           <t>Synnergie</t>
         </is>
       </c>
-      <c r="M32" s="103" t="n"/>
+      <c r="M32" s="103" t="inlineStr">
+        <is>
+          <t>Brett Anderson</t>
+        </is>
+      </c>
       <c r="N32" s="103" t="inlineStr">
         <is>
           <t>Audrey Debaere</t>
         </is>
       </c>
-      <c r="O32" s="103" t="n"/>
+      <c r="O32" s="103" t="inlineStr">
+        <is>
+          <t>Deepak Gudwani</t>
+        </is>
+      </c>
       <c r="P32" s="103" t="inlineStr">
         <is>
           <t>Bhavya Reddy</t>
@@ -13864,13 +13944,23 @@
       <c r="T32" s="104" t="n">
         <v>1625</v>
       </c>
-      <c r="U32" s="99" t="n"/>
-      <c r="V32" s="99" t="n"/>
-      <c r="W32" s="99" t="n"/>
-      <c r="X32" s="99" t="n"/>
+      <c r="U32" s="99" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="V32" s="99" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W32" s="99" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="X32" s="99" t="n">
+        <v>0.6</v>
+      </c>
       <c r="Y32" s="99" t="n"/>
       <c r="Z32" s="99" t="n"/>
-      <c r="AA32" s="105" t="n"/>
+      <c r="AA32" s="105" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AB32" s="105" t="n"/>
       <c r="AC32" s="103" t="n"/>
       <c r="AD32" s="106">
@@ -13931,13 +14021,21 @@
           <t>Synnergie</t>
         </is>
       </c>
-      <c r="M33" s="93" t="n"/>
+      <c r="M33" s="93" t="inlineStr">
+        <is>
+          <t>Brett Anderson</t>
+        </is>
+      </c>
       <c r="N33" s="93" t="inlineStr">
         <is>
           <t>Cristian Varelas</t>
         </is>
       </c>
-      <c r="O33" s="93" t="n"/>
+      <c r="O33" s="93" t="inlineStr">
+        <is>
+          <t>Deepak Gudwani</t>
+        </is>
+      </c>
       <c r="P33" s="93" t="inlineStr">
         <is>
           <t>Sangamesh Koti</t>
@@ -13954,13 +14052,25 @@
       <c r="T33" s="107" t="n">
         <v>260</v>
       </c>
-      <c r="U33" s="89" t="n"/>
-      <c r="V33" s="89" t="n"/>
-      <c r="W33" s="89" t="n"/>
-      <c r="X33" s="89" t="n"/>
-      <c r="Y33" s="89" t="n"/>
+      <c r="U33" s="89" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="V33" s="89" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W33" s="89" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="X33" s="89" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="Y33" s="89" t="n">
+        <v>0.1</v>
+      </c>
       <c r="Z33" s="89" t="n"/>
-      <c r="AA33" s="96" t="n"/>
+      <c r="AA33" s="96" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AB33" s="96" t="n"/>
       <c r="AC33" s="93" t="n"/>
       <c r="AD33" s="108">
@@ -14021,13 +14131,21 @@
           <t>Synnergie</t>
         </is>
       </c>
-      <c r="M34" s="103" t="n"/>
+      <c r="M34" s="103" t="inlineStr">
+        <is>
+          <t>Bettina Kotico</t>
+        </is>
+      </c>
       <c r="N34" s="103" t="inlineStr">
         <is>
           <t>Cristian Varelas</t>
         </is>
       </c>
-      <c r="O34" s="103" t="n"/>
+      <c r="O34" s="103" t="inlineStr">
+        <is>
+          <t>Deepak Gudwani</t>
+        </is>
+      </c>
       <c r="P34" s="103" t="inlineStr">
         <is>
           <t>Vishnu Premen</t>
@@ -14042,13 +14160,27 @@
         <v>120</v>
       </c>
       <c r="T34" s="104" t="n"/>
-      <c r="U34" s="99" t="n"/>
-      <c r="V34" s="99" t="n"/>
-      <c r="W34" s="99" t="n"/>
-      <c r="X34" s="99" t="n"/>
-      <c r="Y34" s="99" t="n"/>
-      <c r="Z34" s="99" t="n"/>
-      <c r="AA34" s="105" t="n"/>
+      <c r="U34" s="99" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="V34" s="99" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W34" s="99" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="X34" s="99" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="Y34" s="99" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Z34" s="99" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AA34" s="105" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AB34" s="105" t="n"/>
       <c r="AC34" s="103" t="inlineStr">
         <is>
@@ -14259,18 +14391,38 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I37" s="314" t="n"/>
-      <c r="J37" s="314" t="n"/>
+      <c r="I37" s="314" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J37" s="314" t="n">
+        <v>46190</v>
+      </c>
       <c r="K37" s="314" t="n"/>
       <c r="L37" s="89" t="inlineStr">
         <is>
           <t>Systems Applications</t>
         </is>
       </c>
-      <c r="M37" s="93" t="n"/>
-      <c r="N37" s="93" t="n"/>
-      <c r="O37" s="93" t="n"/>
-      <c r="P37" s="93" t="n"/>
+      <c r="M37" s="93" t="inlineStr">
+        <is>
+          <t>Emily Fridley</t>
+        </is>
+      </c>
+      <c r="N37" s="93" t="inlineStr">
+        <is>
+          <t>Cristian Varelas</t>
+        </is>
+      </c>
+      <c r="O37" s="93" t="inlineStr">
+        <is>
+          <t>Ajay Kumar</t>
+        </is>
+      </c>
+      <c r="P37" s="93" t="inlineStr">
+        <is>
+          <t>Vishnu Premen</t>
+        </is>
+      </c>
       <c r="R37" s="89" t="inlineStr">
         <is>
           <t>S: &lt; 80 Hours</t>
@@ -14280,13 +14432,25 @@
         <v>40</v>
       </c>
       <c r="T37" s="107" t="n"/>
-      <c r="U37" s="89" t="n"/>
-      <c r="V37" s="89" t="n"/>
-      <c r="W37" s="89" t="n"/>
-      <c r="X37" s="89" t="n"/>
-      <c r="Y37" s="89" t="n"/>
+      <c r="U37" s="89" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="V37" s="89" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W37" s="89" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="X37" s="89" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="Y37" s="89" t="n">
+        <v>0.1</v>
+      </c>
       <c r="Z37" s="89" t="n"/>
-      <c r="AA37" s="96" t="n"/>
+      <c r="AA37" s="96" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AB37" s="96" t="n"/>
       <c r="AC37" s="93" t="n"/>
       <c r="AD37" s="108">
@@ -14347,13 +14511,21 @@
           <t>Synnergie</t>
         </is>
       </c>
-      <c r="M38" s="103" t="n"/>
+      <c r="M38" s="103" t="inlineStr">
+        <is>
+          <t>Brett Anderson</t>
+        </is>
+      </c>
       <c r="N38" s="103" t="inlineStr">
         <is>
           <t>Audrey Debaere</t>
         </is>
       </c>
-      <c r="O38" s="103" t="n"/>
+      <c r="O38" s="103" t="inlineStr">
+        <is>
+          <t>Deepak Gudwani</t>
+        </is>
+      </c>
       <c r="P38" s="103" t="inlineStr">
         <is>
           <t>Sangamesh Koti</t>
@@ -14364,13 +14536,23 @@
         <v>320</v>
       </c>
       <c r="T38" s="104" t="n"/>
-      <c r="U38" s="99" t="n"/>
-      <c r="V38" s="99" t="n"/>
-      <c r="W38" s="99" t="n"/>
-      <c r="X38" s="99" t="n"/>
+      <c r="U38" s="99" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="V38" s="99" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W38" s="99" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="X38" s="99" t="n">
+        <v>0.4</v>
+      </c>
       <c r="Y38" s="99" t="n"/>
       <c r="Z38" s="99" t="n"/>
-      <c r="AA38" s="105" t="n"/>
+      <c r="AA38" s="105" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AB38" s="105" t="n"/>
       <c r="AC38" s="103" t="n"/>
       <c r="AD38" s="106">
@@ -14417,22 +14599,38 @@
           <t>Highest</t>
         </is>
       </c>
-      <c r="I39" s="314" t="n"/>
-      <c r="J39" s="314" t="n"/>
+      <c r="I39" s="314" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J39" s="314" t="n">
+        <v>46253</v>
+      </c>
       <c r="K39" s="314" t="n"/>
       <c r="L39" s="89" t="inlineStr">
         <is>
           <t>Systems Applications</t>
         </is>
       </c>
-      <c r="M39" s="93" t="n"/>
+      <c r="M39" s="93" t="inlineStr">
+        <is>
+          <t>Brett Anderson</t>
+        </is>
+      </c>
       <c r="N39" s="93" t="inlineStr">
         <is>
           <t>Cristian Varelas</t>
         </is>
       </c>
-      <c r="O39" s="93" t="n"/>
-      <c r="P39" s="93" t="n"/>
+      <c r="O39" s="93" t="inlineStr">
+        <is>
+          <t>Deepak Gudwani</t>
+        </is>
+      </c>
+      <c r="P39" s="93" t="inlineStr">
+        <is>
+          <t>Sarath Yeturu</t>
+        </is>
+      </c>
       <c r="R39" s="89" t="inlineStr">
         <is>
           <t>S: &lt; 80 Hours</t>
@@ -14442,13 +14640,23 @@
         <v>40</v>
       </c>
       <c r="T39" s="107" t="n"/>
-      <c r="U39" s="89" t="n"/>
-      <c r="V39" s="89" t="n"/>
-      <c r="W39" s="89" t="n"/>
-      <c r="X39" s="89" t="n"/>
+      <c r="U39" s="89" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="V39" s="89" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W39" s="89" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="X39" s="89" t="n">
+        <v>0.5</v>
+      </c>
       <c r="Y39" s="89" t="n"/>
       <c r="Z39" s="89" t="n"/>
-      <c r="AA39" s="96" t="n"/>
+      <c r="AA39" s="96" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AB39" s="96" t="n"/>
       <c r="AC39" s="93" t="n"/>
       <c r="AD39" s="108">
@@ -14495,8 +14703,12 @@
           <t>Highest</t>
         </is>
       </c>
-      <c r="I40" s="315" t="n"/>
-      <c r="J40" s="315" t="n"/>
+      <c r="I40" s="315" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J40" s="315" t="n">
+        <v>46274</v>
+      </c>
       <c r="K40" s="315" t="n"/>
       <c r="L40" s="99" t="inlineStr">
         <is>
@@ -14513,8 +14725,16 @@
           <t>Audrey Debaere</t>
         </is>
       </c>
-      <c r="O40" s="103" t="n"/>
-      <c r="P40" s="103" t="n"/>
+      <c r="O40" s="103" t="inlineStr">
+        <is>
+          <t>Deepak Gudwani</t>
+        </is>
+      </c>
+      <c r="P40" s="103" t="inlineStr">
+        <is>
+          <t>Bhavya Reddy</t>
+        </is>
+      </c>
       <c r="Q40" t="inlineStr">
         <is>
           <t>Alex Young</t>
@@ -14529,13 +14749,25 @@
         <v>80</v>
       </c>
       <c r="T40" s="104" t="n"/>
-      <c r="U40" s="99" t="n"/>
-      <c r="V40" s="99" t="n"/>
-      <c r="W40" s="99" t="n"/>
-      <c r="X40" s="99" t="n"/>
-      <c r="Y40" s="99" t="n"/>
+      <c r="U40" s="99" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="V40" s="99" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W40" s="99" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="X40" s="99" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Y40" s="99" t="n">
+        <v>0.2</v>
+      </c>
       <c r="Z40" s="99" t="n"/>
-      <c r="AA40" s="105" t="n"/>
+      <c r="AA40" s="105" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AB40" s="105" t="n"/>
       <c r="AC40" s="103" t="n"/>
       <c r="AD40" s="106">
@@ -14582,22 +14814,38 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I41" s="314" t="n"/>
-      <c r="J41" s="314" t="n"/>
+      <c r="I41" s="314" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J41" s="314" t="n">
+        <v>46141</v>
+      </c>
       <c r="K41" s="314" t="n"/>
       <c r="L41" s="89" t="inlineStr">
         <is>
           <t>Synnergie</t>
         </is>
       </c>
-      <c r="M41" s="93" t="n"/>
+      <c r="M41" s="93" t="inlineStr">
+        <is>
+          <t>Bettina Kotico</t>
+        </is>
+      </c>
       <c r="N41" s="93" t="inlineStr">
         <is>
           <t>Audrey Debaere</t>
         </is>
       </c>
-      <c r="O41" s="93" t="n"/>
-      <c r="P41" s="93" t="n"/>
+      <c r="O41" s="93" t="inlineStr">
+        <is>
+          <t>Deepak Gudwani</t>
+        </is>
+      </c>
+      <c r="P41" s="93" t="inlineStr">
+        <is>
+          <t>Vishnu Premen</t>
+        </is>
+      </c>
       <c r="R41" s="89" t="inlineStr">
         <is>
           <t>L: 160-320 Hours</t>
@@ -14607,13 +14855,25 @@
         <v>320</v>
       </c>
       <c r="T41" s="107" t="n"/>
-      <c r="U41" s="89" t="n"/>
-      <c r="V41" s="89" t="n"/>
-      <c r="W41" s="89" t="n"/>
-      <c r="X41" s="89" t="n"/>
-      <c r="Y41" s="89" t="n"/>
+      <c r="U41" s="89" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="V41" s="89" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W41" s="89" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="X41" s="89" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="Y41" s="89" t="n">
+        <v>0.1</v>
+      </c>
       <c r="Z41" s="89" t="n"/>
-      <c r="AA41" s="96" t="n"/>
+      <c r="AA41" s="96" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AB41" s="96" t="n"/>
       <c r="AC41" s="93" t="n"/>
       <c r="AD41" s="108">
@@ -14682,7 +14942,11 @@
           <t>Audrey Debaere</t>
         </is>
       </c>
-      <c r="O42" s="114" t="n"/>
+      <c r="O42" s="114" t="inlineStr">
+        <is>
+          <t>Deepak Gudwani</t>
+        </is>
+      </c>
       <c r="P42" s="114" t="inlineStr">
         <is>
           <t>Alex Young</t>
@@ -14702,13 +14966,25 @@
         <v>40</v>
       </c>
       <c r="T42" s="115" t="n"/>
-      <c r="U42" s="111" t="n"/>
-      <c r="V42" s="111" t="n"/>
-      <c r="W42" s="111" t="n"/>
-      <c r="X42" s="111" t="n"/>
+      <c r="U42" s="111" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="V42" s="111" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W42" s="111" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="X42" s="111" t="n">
+        <v>0.6</v>
+      </c>
       <c r="Y42" s="111" t="n"/>
-      <c r="Z42" s="111" t="n"/>
-      <c r="AA42" s="116" t="n"/>
+      <c r="Z42" s="111" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AA42" s="116" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AB42" s="116" t="n"/>
       <c r="AC42" s="114" t="n"/>
       <c r="AD42" s="118">
@@ -14759,7 +15035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -15981,6 +16257,8 @@
         <v/>
       </c>
     </row>
+    <row r="28"/>
+    <row r="29"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="1" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0"/>
   <autoFilter ref="A3:K27"/>

</xml_diff>